<commit_message>
chore: refresh SAT cache + report (2026-05-12)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evol_Estado" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evol_Cadena" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Evol_Estado" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Evol_Cadena" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -737,43 +737,43 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>10</v>
@@ -782,7 +782,7 @@
         <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -806,49 +806,49 @@
         <v>1</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>5</v>
@@ -871,46 +871,52 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -931,25 +937,35 @@
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O8" s="4" t="inlineStr"/>
       <c r="P8" s="4" t="inlineStr"/>
       <c r="Q8" s="4" t="inlineStr"/>
       <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T8" s="4" t="inlineStr"/>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -969,7 +985,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
@@ -978,19 +994,19 @@
         <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
@@ -1005,10 +1021,10 @@
         <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1029,15 +1045,21 @@
       <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="4" t="inlineStr"/>
       <c r="P10" s="4" t="inlineStr"/>
-      <c r="Q10" s="4" t="inlineStr"/>
-      <c r="R10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="4" t="inlineStr"/>
       <c r="T10" s="4" t="n">
         <v>1</v>
@@ -1046,7 +1068,7 @@
         <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1088,7 +1110,7 @@
         <v>4</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>4</v>
@@ -1112,10 +1134,10 @@
         <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>8</v>
@@ -1124,7 +1146,7 @@
         <v>13</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1142,26 +1164,56 @@
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
-      <c r="Q12" s="4" t="inlineStr"/>
-      <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1190,17 +1242,21 @@
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="6" t="inlineStr"/>
       <c r="Q13" s="6" t="inlineStr"/>
-      <c r="R13" s="6" t="inlineStr"/>
-      <c r="S13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="T13" s="6" t="inlineStr"/>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1254,16 +1310,16 @@
         <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -1300,13 +1356,13 @@
         <v>6</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>13</v>
       </c>
       <c r="W15" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
@@ -1349,7 +1405,7 @@
         <v>2</v>
       </c>
       <c r="W16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1360,7 +1416,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Enviado a técnico externo</t>
+          <t>Esperando respuesta cliente a presupuesto</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr"/>
@@ -1368,124 +1424,159 @@
       <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="6" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O17" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T17" s="6" t="n">
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Externa</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Enviado a técnico externo</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T18" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="U17" s="6" t="n">
+      <c r="U18" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="V17" s="6" t="n">
+      <c r="V18" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="W17" s="6" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr"/>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="W18" s="4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Total abiertas</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="8" t="n">
+      <c r="C19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F19" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="G18" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="H18" s="8" t="n">
+      <c r="G19" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="P19" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q19" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="I18" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="J18" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="L18" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="M18" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="N18" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="O18" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="P18" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q18" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="R18" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="S18" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="T18" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="U18" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="V18" s="8" t="n">
+      <c r="R19" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="S19" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="T19" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="U19" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="W18" s="8" t="n">
-        <v>100</v>
+      <c r="V19" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="W19" s="8" t="n">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1666,49 +1757,49 @@
         <v>3</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>14</v>
@@ -1732,52 +1823,52 @@
         <v>1</v>
       </c>
       <c r="G5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -1790,28 +1881,56 @@
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" s="4" t="inlineStr"/>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1962,49 +2081,49 @@
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>4</v>
@@ -2032,52 +2151,52 @@
         <v>2</v>
       </c>
       <c r="G11" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="H11" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="N11" s="10" t="n">
+      <c r="P11" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>9</v>
-      </c>
       <c r="Q11" s="10" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -2099,55 +2218,55 @@
         <v>7</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G12" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="H12" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>22</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-13)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-12</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-13</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -673,46 +673,46 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="R4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -745,43 +745,43 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
+      <c r="R5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>12</v>
@@ -811,43 +811,43 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>5</v>
@@ -883,46 +883,46 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="M7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="Q7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="S7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -951,41 +951,41 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>1</v>
@@ -1021,46 +1021,46 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="T9" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1093,44 +1093,44 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1163,46 +1163,46 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="U11" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1238,43 +1238,43 @@
         <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1307,44 +1307,44 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1377,46 +1377,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="Q14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R14" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1447,41 +1447,41 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>12</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O15" s="6" t="n">
+      <c r="P15" s="6" t="inlineStr"/>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q15" s="6" t="inlineStr"/>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>22</v>
@@ -1517,7 +1517,9 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1536,9 +1538,7 @@
       <c r="R16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
@@ -1573,43 +1573,43 @@
         <v>6</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>3</v>
@@ -1649,27 +1649,27 @@
         <v>3</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1707,46 +1707,46 @@
         <v>24</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>16</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
@@ -1775,43 +1775,43 @@
         <v>129</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="P20" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="S20" s="8" t="n">
         <v>102</v>
       </c>
       <c r="T20" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="U20" s="8" t="n">
         <v>102</v>
-      </c>
-      <c r="U20" s="8" t="n">
-        <v>96</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>102</v>
@@ -1860,7 +1860,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-12</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-13</t>
         </is>
       </c>
     </row>
@@ -1902,72 +1902,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -1996,40 +1996,40 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="R4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>14</v>
@@ -2066,37 +2066,37 @@
         <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>22</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>23</v>
@@ -2136,13 +2136,13 @@
         <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>6</v>
@@ -2151,22 +2151,22 @@
         <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2199,7 +2199,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>2</v>
@@ -2208,7 +2208,7 @@
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>1</v>
@@ -2260,43 +2260,43 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
@@ -2339,17 +2339,17 @@
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -2391,7 +2391,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
@@ -2409,13 +2409,13 @@
         <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
@@ -2424,7 +2424,7 @@
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2455,43 +2455,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>47</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="Q11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>46</v>
@@ -2522,43 +2522,43 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="S12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>102</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>96</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>102</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-14)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-13</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="Q4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -745,43 +745,43 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="P5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>12</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>18</v>
@@ -811,43 +811,43 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -883,43 +883,43 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="N7" s="6" t="n">
+      <c r="P7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="R7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -951,41 +951,41 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
@@ -1021,43 +1021,43 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="S9" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>4</v>
@@ -1096,38 +1096,38 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>3</v>
@@ -1163,43 +1163,43 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>10</v>
@@ -1235,43 +1235,43 @@
         <v>5</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>4</v>
@@ -1307,41 +1307,41 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="Q13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>6</v>
@@ -1377,43 +1377,43 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="P14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="R14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>5</v>
@@ -1447,38 +1447,38 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>12</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N15" s="6" t="n">
+      <c r="O15" s="6" t="inlineStr"/>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P15" s="6" t="inlineStr"/>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>22</v>
@@ -1516,7 +1516,9 @@
       </c>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1535,9 +1537,7 @@
       <c r="Q16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
@@ -1573,43 +1573,43 @@
         <v>6</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>4</v>
@@ -1646,32 +1646,32 @@
         <v>3</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V18" s="4" t="n">
         <v>2</v>
@@ -1707,40 +1707,40 @@
         <v>24</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>16</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>15</v>
@@ -1775,43 +1775,43 @@
         <v>129</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="P20" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="R20" s="8" t="n">
         <v>102</v>
       </c>
       <c r="S20" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="T20" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="T20" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="U20" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>106</v>
@@ -1860,7 +1860,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-13</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -1902,72 +1902,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -1996,43 +1996,43 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>17</v>
@@ -2063,43 +2063,43 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>22</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>24</v>
@@ -2133,13 +2133,13 @@
         <v>5</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>6</v>
@@ -2148,22 +2148,22 @@
         <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
@@ -2196,7 +2196,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
@@ -2205,7 +2205,7 @@
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>1</v>
@@ -2260,40 +2260,40 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
@@ -2336,17 +2336,17 @@
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2354,10 +2354,10 @@
         <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
@@ -2388,7 +2388,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>4</v>
@@ -2406,13 +2406,13 @@
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>4</v>
@@ -2421,7 +2421,7 @@
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
@@ -2455,43 +2455,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>47</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="P11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>47</v>
@@ -2522,43 +2522,43 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="R12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="S12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>106</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-15)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-14</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>4</v>
@@ -745,43 +745,43 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>13</v>
@@ -811,40 +811,40 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -883,43 +883,43 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="M7" s="6" t="n">
+      <c r="O7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="Q7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>4</v>
@@ -951,41 +951,41 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>1</v>
@@ -1021,43 +1021,43 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="R9" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>6</v>
@@ -1093,41 +1093,41 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>1</v>
@@ -1163,43 +1163,43 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>11</v>
@@ -1235,46 +1235,46 @@
         <v>5</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1310,41 +1310,41 @@
         <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="P13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -1377,46 +1377,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="Q14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V14" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V14" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1447,41 +1447,41 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M15" s="6" t="n">
+      <c r="N15" s="6" t="inlineStr"/>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O15" s="6" t="inlineStr"/>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="S15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>19</v>
@@ -1515,7 +1515,9 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1534,9 +1536,7 @@
       <c r="P16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
@@ -1576,37 +1576,37 @@
         <v>3</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>4</v>
@@ -1643,32 +1643,32 @@
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U18" s="4" t="n">
         <v>2</v>
@@ -1707,43 +1707,43 @@
         <v>24</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>16</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>15</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>11</v>
@@ -1775,43 +1775,43 @@
         <v>129</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P20" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="Q20" s="8" t="n">
         <v>102</v>
       </c>
       <c r="R20" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S20" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="S20" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="T20" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>99</v>
@@ -1860,7 +1860,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-14</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -1902,72 +1902,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -1996,40 +1996,40 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>17</v>
@@ -2063,40 +2063,40 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>22</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>24</v>
@@ -2130,13 +2130,13 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>6</v>
@@ -2145,28 +2145,28 @@
         <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2193,7 +2193,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>2</v>
@@ -2202,7 +2202,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>1</v>
@@ -2263,40 +2263,40 @@
         <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="N8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>6</v>
@@ -2333,17 +2333,17 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2351,14 +2351,12 @@
         <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2401,13 +2399,13 @@
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>4</v>
@@ -2416,13 +2414,13 @@
         <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>3</v>
@@ -2453,43 +2451,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>47</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>45</v>
@@ -2520,43 +2518,43 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="P12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="Q12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="R12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>99</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-16)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-15</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-16</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-15</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-17)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-16</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-17</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-16</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-18)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-17</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -673,46 +673,46 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -745,43 +745,43 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -811,43 +811,43 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>8</v>
@@ -883,43 +883,43 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="M7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="N7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="P7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>3</v>
@@ -954,35 +954,35 @@
         <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="P8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>1</v>
@@ -1021,43 +1021,43 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="Q9" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -1095,39 +1095,39 @@
       <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1163,40 +1163,40 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>11</v>
@@ -1235,43 +1235,43 @@
         <v>5</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
@@ -1307,41 +1307,41 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O13" s="6" t="inlineStr"/>
+      <c r="P13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
@@ -1377,43 +1377,43 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>5</v>
@@ -1450,38 +1450,38 @@
         <v>12</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L15" s="6" t="n">
+      <c r="M15" s="6" t="inlineStr"/>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N15" s="6" t="inlineStr"/>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>20</v>
@@ -1514,7 +1514,9 @@
       <c r="H16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1533,9 +1535,7 @@
       <c r="O16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
@@ -1573,43 +1573,43 @@
         <v>6</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>1</v>
@@ -1643,36 +1643,34 @@
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="U18" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1705,43 +1703,43 @@
         <v>24</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>16</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>15</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>26</v>
@@ -1773,46 +1771,46 @@
         <v>129</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="P20" s="8" t="n">
         <v>102</v>
       </c>
       <c r="Q20" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R20" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="R20" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="S20" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="V20" s="8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1858,7 +1856,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-17</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -1900,72 +1898,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -1994,43 +1992,43 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>25</v>
@@ -2064,40 +2062,40 @@
         <v>22</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>23</v>
@@ -2128,10 +2126,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>6</v>
@@ -2140,31 +2138,31 @@
         <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>2</v>
@@ -2197,7 +2195,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>1</v>
@@ -2258,46 +2256,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -2328,17 +2326,17 @@
         <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2346,15 +2344,15 @@
         <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2396,13 +2394,13 @@
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>4</v>
@@ -2411,13 +2409,13 @@
         <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>3</v>
@@ -2451,43 +2449,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>47</v>
-      </c>
       <c r="J11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="N11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>41</v>
@@ -2518,46 +2516,46 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="P12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="Q12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="R12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-19)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-18</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -673,40 +673,40 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>5</v>
@@ -745,40 +745,40 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
@@ -811,43 +811,43 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>7</v>
@@ -883,44 +883,42 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="M7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="O7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -949,42 +947,40 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="P8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U8" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U8" s="4" t="inlineStr"/>
       <c r="V8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1017,46 +1013,46 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N9" s="6" t="n">
+      <c r="P9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="Q9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="R9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="T9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="V9" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="U9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1088,45 +1084,45 @@
       <c r="H10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1159,43 +1155,43 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>9</v>
@@ -1234,37 +1230,37 @@
         <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O12" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>2</v>
@@ -1303,44 +1299,44 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1373,46 +1369,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>11</v>
-      </c>
       <c r="N14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O14" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U14" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="V14" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1443,41 +1439,41 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K15" s="6" t="n">
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M15" s="6" t="inlineStr"/>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>12</v>
@@ -1528,15 +1524,15 @@
       <c r="N16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1579,9 +1575,7 @@
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
@@ -1622,7 +1616,9 @@
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1638,9 +1634,7 @@
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1710,43 +1704,43 @@
         <v>5</v>
       </c>
       <c r="J20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="M20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1776,34 +1770,32 @@
         <v>3</v>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="T21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
     </row>
@@ -1840,43 +1832,43 @@
         <v>16</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23">
@@ -1905,43 +1897,43 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="P23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="Q23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="R23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>89</v>
@@ -1990,7 +1982,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-18</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2032,72 +2024,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2126,43 +2118,43 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>21</v>
@@ -2193,43 +2185,43 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>21</v>
@@ -2260,7 +2252,7 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>6</v>
@@ -2269,34 +2261,34 @@
         <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2326,7 +2318,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
@@ -2390,43 +2382,43 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>14</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
@@ -2457,17 +2449,17 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2475,15 +2467,15 @@
         <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2525,28 +2517,28 @@
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>3</v>
@@ -2583,43 +2575,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>32</v>
@@ -2650,43 +2642,43 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="O12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="P12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>89</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-20)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-19</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="R4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>6</v>
@@ -745,37 +745,37 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>14</v>
@@ -811,43 +811,43 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>9</v>
@@ -883,41 +883,39 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="K7" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="L7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
     </row>
@@ -947,40 +945,40 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="N8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="O8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr"/>
+      <c r="U8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V8" s="4" t="n">
         <v>1</v>
       </c>
@@ -1015,46 +1013,46 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M9" s="6" t="n">
+      <c r="O9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="P9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1086,45 +1084,47 @@
       <c r="H10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1157,43 +1157,43 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>10</v>
@@ -1229,46 +1229,46 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N12" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1301,44 +1301,44 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1371,43 +1371,43 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>11</v>
-      </c>
       <c r="M14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N14" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>3</v>
@@ -1441,41 +1441,41 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="P15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>14</v>
@@ -1523,18 +1523,16 @@
       <c r="M16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
-      <c r="T16" s="4" t="inlineStr"/>
-      <c r="U16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1572,9 +1570,7 @@
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
@@ -1615,7 +1611,9 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1631,9 +1629,7 @@
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
@@ -1701,43 +1697,43 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="L20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>4</v>
@@ -1771,30 +1767,30 @@
       </c>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="S21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
@@ -1829,43 +1825,43 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>27</v>
@@ -1897,43 +1893,43 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="N23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="O23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="P23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="P23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="Q23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>97</v>
@@ -1982,7 +1978,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-19</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -2024,72 +2020,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -2118,40 +2114,40 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>21</v>
@@ -2185,43 +2181,43 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>22</v>
-      </c>
       <c r="J5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>19</v>
@@ -2258,37 +2254,37 @@
         <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2315,7 +2311,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>1</v>
@@ -2382,43 +2378,43 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>9</v>
@@ -2451,12 +2447,12 @@
       <c r="H9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2464,15 +2460,15 @@
         <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2514,28 +2510,28 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>3</v>
@@ -2544,7 +2540,7 @@
         <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2575,43 +2571,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>38</v>
@@ -2642,43 +2638,43 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>97</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-21)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,13 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-20</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -642,6 +643,11 @@
           <t>2026-05-20</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -714,6 +720,9 @@
       <c r="V4" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="W4" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -784,6 +793,9 @@
         <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="W5" s="6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -852,6 +864,9 @@
       <c r="V6" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="W6" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -920,6 +935,9 @@
       <c r="V7" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="W7" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -984,6 +1002,9 @@
       <c r="V8" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="W8" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1056,6 +1077,9 @@
       <c r="V9" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="W9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1128,6 +1152,9 @@
       <c r="V10" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W10" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1200,6 +1227,9 @@
       <c r="V11" s="6" t="n">
         <v>10</v>
       </c>
+      <c r="W11" s="6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1272,6 +1302,9 @@
       <c r="V12" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="W12" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1342,6 +1375,9 @@
       <c r="V13" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="W13" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1412,6 +1448,9 @@
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="W14" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1480,6 +1519,9 @@
         <v>14</v>
       </c>
       <c r="V15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1536,6 +1578,7 @@
       </c>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1584,6 +1627,7 @@
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
+      <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1634,6 +1678,7 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1668,6 +1713,7 @@
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
+      <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1738,6 +1784,9 @@
         <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="W20" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1796,6 +1845,7 @@
       <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
+      <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1866,6 +1916,9 @@
         <v>27</v>
       </c>
       <c r="V22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1936,10 +1989,13 @@
       <c r="V23" s="8" t="n">
         <v>94</v>
       </c>
+      <c r="W23" s="8" t="n">
+        <v>94</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1951,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1975,12 +2031,13 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-20</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -2090,6 +2147,11 @@
           <t>2026-05-20</t>
         </is>
       </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2157,6 +2219,9 @@
       <c r="U4" s="4" t="n">
         <v>20</v>
       </c>
+      <c r="V4" s="4" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2224,6 +2289,9 @@
       <c r="U5" s="6" t="n">
         <v>18</v>
       </c>
+      <c r="V5" s="6" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2291,6 +2359,9 @@
       <c r="U6" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="V6" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2354,6 +2425,9 @@
       <c r="U7" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="V7" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2419,6 +2493,9 @@
         <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2480,6 +2557,9 @@
       <c r="U9" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="V9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2547,6 +2627,9 @@
       <c r="U10" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="V10" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2614,6 +2697,9 @@
       <c r="U11" s="10" t="n">
         <v>37</v>
       </c>
+      <c r="V11" s="10" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2681,10 +2767,13 @@
       <c r="U12" s="8" t="n">
         <v>94</v>
       </c>
+      <c r="V12" s="8" t="n">
+        <v>94</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-22)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-21</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -679,40 +679,40 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>6</v>
@@ -754,34 +754,34 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>14</v>
@@ -790,10 +790,10 @@
         <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>14</v>
@@ -823,46 +823,46 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>6</v>
@@ -898,43 +898,41 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="M7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
-      <c r="V7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="U7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -963,42 +961,42 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="N8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>3</v>
@@ -1040,37 +1038,37 @@
         <v>7</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="O9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="P9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
@@ -1109,46 +1107,46 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>1</v>
@@ -1187,37 +1185,37 @@
         <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>10</v>
@@ -1259,49 +1257,49 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1334,47 +1332,47 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1407,46 +1405,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>11</v>
-      </c>
       <c r="L14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>3</v>
@@ -1480,44 +1478,44 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K15" s="6" t="inlineStr"/>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="O15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>16</v>
@@ -1562,18 +1560,16 @@
       <c r="L16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="inlineStr"/>
-      <c r="T16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
@@ -1610,9 +1606,7 @@
       <c r="I17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
@@ -1654,7 +1648,9 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1670,9 +1666,7 @@
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1743,46 +1737,46 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>4</v>
@@ -1815,30 +1809,30 @@
         <v>3</v>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr"/>
+      <c r="N21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="R21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
@@ -1875,46 +1869,46 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="S22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="T22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="V22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>20</v>
@@ -1946,46 +1940,46 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="M23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="N23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="O23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="O23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="P23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>88</v>
@@ -2035,7 +2029,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-21</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -2077,77 +2071,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -2176,46 +2170,46 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>17</v>
@@ -2246,46 +2240,46 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>19</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>19</v>
@@ -2319,43 +2313,43 @@
         <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2452,46 +2446,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -2521,12 +2515,12 @@
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2534,15 +2528,15 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2587,13 +2581,13 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>4</v>
@@ -2602,13 +2596,13 @@
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>3</v>
@@ -2617,13 +2611,13 @@
         <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -2654,46 +2648,46 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>46</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="T11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>38</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>37</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>38</v>
@@ -2724,46 +2718,46 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="O12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>88</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-23)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-22</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-23</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-22</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-24)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-23</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-23</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-25)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-24</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -679,37 +679,37 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>6</v>
@@ -718,7 +718,7 @@
         <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -754,31 +754,31 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
+      <c r="M5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>14</v>
@@ -787,13 +787,13 @@
         <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="U5" s="6" t="n">
+      <c r="V5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>13</v>
@@ -826,43 +826,43 @@
         <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="S6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="U6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>9</v>
@@ -898,40 +898,38 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="T7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
@@ -961,45 +959,45 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1035,46 +1033,46 @@
         <v>7</v>
       </c>
       <c r="J9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="O9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="P9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="S9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1107,43 +1105,43 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>1</v>
@@ -1182,37 +1180,37 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>10</v>
@@ -1221,7 +1219,7 @@
         <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>6</v>
@@ -1257,49 +1255,49 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1335,44 +1333,44 @@
         <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1405,46 +1403,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>2</v>
@@ -1477,45 +1475,45 @@
       <c r="H15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="I15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>11</v>
@@ -1557,18 +1555,16 @@
       <c r="K16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
-      <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
@@ -1603,9 +1599,7 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1647,7 +1641,9 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1663,9 +1659,7 @@
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
@@ -1737,49 +1731,49 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1815,23 +1809,21 @@
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="Q21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
@@ -1869,46 +1861,46 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="P22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V22" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>15</v>
@@ -1940,49 +1932,49 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="M23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="N23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="N23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="O23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2029,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-24</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -2071,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -2170,46 +2162,46 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>16</v>
@@ -2240,46 +2232,46 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>16</v>
@@ -2310,49 +2302,49 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2446,46 +2438,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
@@ -2517,7 +2509,9 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2525,15 +2519,15 @@
         <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2578,13 +2572,13 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
@@ -2593,13 +2587,13 @@
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>3</v>
@@ -2608,16 +2602,16 @@
         <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2648,49 +2642,49 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="T11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="U11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
@@ -2718,49 +2712,49 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="N12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-26)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-25</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -679,34 +679,34 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>6</v>
@@ -715,7 +715,7 @@
         <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -754,28 +754,28 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>14</v>
@@ -784,16 +784,16 @@
         <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="U5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>11</v>
@@ -823,46 +823,46 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="R6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="V6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>12</v>
@@ -898,42 +898,40 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="S7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
-      <c r="V7" s="6" t="inlineStr"/>
-      <c r="W7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="V7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -961,45 +959,45 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1032,49 +1030,49 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="K9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="N9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="R9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1110,46 +1108,46 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1182,34 +1180,34 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>10</v>
@@ -1218,7 +1216,7 @@
         <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>6</v>
@@ -1260,43 +1258,43 @@
         <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>3</v>
@@ -1332,41 +1330,41 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
@@ -1405,46 +1403,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>1</v>
@@ -1477,45 +1475,47 @@
       <c r="H15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>11</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>13</v>
@@ -1554,18 +1554,16 @@
       <c r="J16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="4" t="inlineStr"/>
-      <c r="R16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
@@ -1642,7 +1640,9 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1658,9 +1658,7 @@
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
@@ -1733,49 +1731,49 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1808,23 +1806,21 @@
       <c r="I21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="P21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
@@ -1863,49 +1859,49 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="P22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="V22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23">
@@ -1934,46 +1930,46 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="K23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="L23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="M23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="M23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="N23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>84</v>
@@ -2023,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-25</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -2065,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -2164,46 +2160,46 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>15</v>
@@ -2234,46 +2230,46 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>26</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -2307,43 +2303,43 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2440,46 +2436,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>10</v>
@@ -2510,7 +2506,9 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2518,15 +2516,15 @@
         <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2543,7 +2541,7 @@
         <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2577,7 +2575,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
@@ -2586,13 +2584,13 @@
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>3</v>
@@ -2601,16 +2599,16 @@
         <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>6</v>
@@ -2644,43 +2642,43 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="S11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>30</v>
@@ -2714,46 +2712,46 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="M12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>84</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-27)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-26</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="N4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>6</v>
@@ -754,25 +754,25 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>14</v>
@@ -781,16 +781,16 @@
         <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="S5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -823,46 +823,46 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="Q6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="S6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>15</v>
@@ -898,39 +898,37 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="R7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
-      <c r="V7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="U7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -958,43 +956,43 @@
       <c r="H8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>1</v>
@@ -1030,46 +1028,46 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="M9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="Q9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>2</v>
@@ -1105,46 +1103,46 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="V10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>5</v>
@@ -1180,31 +1178,31 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>10</v>
@@ -1213,7 +1211,7 @@
         <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>6</v>
@@ -1255,49 +1253,49 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1329,39 +1327,39 @@
       <c r="H13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>3</v>
@@ -1370,7 +1368,7 @@
         <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1403,43 +1401,43 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1476,46 +1474,46 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="T15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>15</v>
@@ -1551,18 +1549,16 @@
       <c r="I16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
@@ -1612,7 +1608,9 @@
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
-      <c r="V17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1641,7 +1639,9 @@
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1657,9 +1657,7 @@
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
@@ -1733,46 +1731,46 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2</v>
@@ -1805,23 +1803,21 @@
         <v>3</v>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="O21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
@@ -1861,46 +1857,46 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="O22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="U22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>14</v>
@@ -1932,46 +1928,46 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="J23" s="8" t="n">
         <v>102</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="L23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="M23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>86</v>
@@ -2021,7 +2017,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-26</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2059,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2158,46 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>19</v>
@@ -2235,43 +2231,43 @@
         <v>26</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="S5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>18</v>
@@ -2302,43 +2298,43 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>2</v>
@@ -2438,46 +2434,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>9</v>
@@ -2507,7 +2503,9 @@
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2515,15 +2513,15 @@
         <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2540,7 +2538,7 @@
         <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2574,40 +2572,40 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>6</v>
@@ -2644,46 +2642,46 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>28</v>
@@ -2714,46 +2712,46 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>102</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="K12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="L12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>86</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-28)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-27</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>10</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="M4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -754,22 +754,22 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>14</v>
@@ -778,22 +778,22 @@
         <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>6</v>
@@ -823,46 +823,46 @@
         <v>10</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="P6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="R6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>20</v>
@@ -898,36 +898,34 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="Q7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="T7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
@@ -956,46 +954,48 @@
       <c r="H8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1028,49 +1028,49 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="P9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1103,46 +1103,46 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>7</v>
@@ -1181,25 +1181,25 @@
         <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>10</v>
@@ -1208,7 +1208,7 @@
         <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>6</v>
@@ -1253,46 +1253,46 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>1</v>
@@ -1327,45 +1327,47 @@
       <c r="H13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V13" s="6" t="n">
         <v>5</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V13" s="6" t="n">
-        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>5</v>
@@ -1401,46 +1403,46 @@
         <v>6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N14" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>2</v>
@@ -1474,46 +1476,46 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>7</v>
@@ -1546,18 +1548,16 @@
       <c r="H16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
@@ -1607,7 +1607,9 @@
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
-      <c r="U17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1638,7 +1640,9 @@
         <v>1</v>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1654,9 +1658,7 @@
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
@@ -1731,43 +1733,43 @@
         <v>6</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1804,19 +1806,19 @@
       </c>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
@@ -1860,40 +1862,40 @@
         <v>11</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="N22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="T22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>14</v>
@@ -1931,43 +1933,43 @@
         <v>102</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="K23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="L23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>80</v>
@@ -2017,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-27</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2059,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2158,46 +2160,46 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>18</v>
@@ -2228,43 +2230,43 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>18</v>
@@ -2298,40 +2300,40 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>2</v>
@@ -2402,9 +2404,7 @@
       <c r="T7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2432,46 +2432,46 @@
         <v>14</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="R8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S8" s="4" t="n">
+      <c r="U8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
@@ -2508,15 +2508,15 @@
         <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
@@ -2576,31 +2576,31 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>6</v>
@@ -2609,7 +2609,7 @@
         <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>8</v>
@@ -2643,43 +2643,43 @@
         <v>43</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="R11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>24</v>
@@ -2713,43 +2713,43 @@
         <v>102</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-29)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-28</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -682,40 +682,40 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="L4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -754,19 +754,19 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>14</v>
@@ -775,25 +775,25 @@
         <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>8</v>
@@ -826,43 +826,43 @@
         <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>16</v>
@@ -898,35 +898,35 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="P7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="S7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
-      <c r="V7" s="6" t="inlineStr"/>
+      <c r="V7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="W7" s="6" t="n">
         <v>7</v>
       </c>
@@ -957,44 +957,44 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>1</v>
@@ -1030,46 +1030,46 @@
         <v>7</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>2</v>
@@ -1105,46 +1105,46 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>3</v>
@@ -1180,25 +1180,25 @@
         <v>7</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>10</v>
@@ -1207,7 +1207,7 @@
         <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>6</v>
@@ -1219,7 +1219,7 @@
         <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1255,49 +1255,49 @@
         <v>4</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1330,49 +1330,49 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="M13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1408,40 +1408,40 @@
         <v>6</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M14" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1478,46 +1478,46 @@
         <v>13</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="S15" s="6" t="n">
+      <c r="T15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>11</v>
@@ -1555,10 +1555,10 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
@@ -1608,7 +1608,9 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
-      <c r="T17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1657,9 +1659,7 @@
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -1738,37 +1738,37 @@
         <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
@@ -1807,19 +1807,19 @@
         <v>3</v>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
@@ -1861,46 +1861,46 @@
         <v>24</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="R22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="M22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="S22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>13</v>
@@ -1932,46 +1932,46 @@
         <v>129</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J23" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="K23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>85</v>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-28</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2162,43 +2162,43 @@
         <v>33</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2232,46 +2232,46 @@
         <v>22</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>19</v>
@@ -2302,37 +2302,37 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>2</v>
@@ -2341,7 +2341,7 @@
         <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>3</v>
@@ -2403,10 +2403,10 @@
       <c r="S7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2439,40 +2439,40 @@
         <v>6</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
@@ -2509,15 +2509,15 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
@@ -2577,31 +2577,31 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
@@ -2610,10 +2610,10 @@
         <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>7</v>
@@ -2644,46 +2644,46 @@
         <v>48</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="Q11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>27</v>
@@ -2714,46 +2714,46 @@
         <v>129</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="I12" s="8" t="n">
         <v>102</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="J12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>85</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-30)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-29</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-29</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-05-31)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-30</t>
+          <t>Evolución abiertas SAT por estado — 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-30</t>
+          <t>Evolución abiertas SAT por cadena — 2026-05-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-01)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-05-31</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -545,107 +545,107 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -661,40 +661,40 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>10</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>6</v>
@@ -703,25 +703,25 @@
         <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="U4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="W4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -736,34 +736,34 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="G5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>14</v>
@@ -772,28 +772,28 @@
         <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>5</v>
@@ -812,57 +812,59 @@
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="n">
+        <v>13</v>
+      </c>
       <c r="F6" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="N6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="P6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="R6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>23</v>
@@ -880,52 +882,52 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="O7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="R7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="V7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>10</v>
@@ -943,55 +945,55 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="G8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>1</v>
@@ -1012,68 +1014,66 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="F9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="H9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="6" t="n">
+      <c r="L9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="W9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="W9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1087,67 +1087,67 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1162,40 +1162,40 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>10</v>
@@ -1204,7 +1204,7 @@
         <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>6</v>
@@ -1216,10 +1216,10 @@
         <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>9</v>
@@ -1237,68 +1237,66 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="W12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1312,49 +1310,49 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="L13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>3</v>
@@ -1363,16 +1361,16 @@
         <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1387,64 +1385,64 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="L14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="N14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>5</v>
@@ -1462,59 +1460,59 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="F15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="G15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="n">
+        <v>13</v>
+      </c>
       <c r="H15" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>22</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R15" s="6" t="n">
+      <c r="S15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>11</v>
@@ -1534,30 +1532,30 @@
           <t>Pendiente agendar llamada (online)</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="D16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -1586,13 +1584,13 @@
         <v>1</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>1</v>
@@ -1607,7 +1605,9 @@
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
-      <c r="S17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1632,17 +1632,17 @@
           <t>En reparación (online)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="n">
         <v>1</v>
@@ -1656,9 +1656,7 @@
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
@@ -1681,10 +1679,10 @@
           <t>Pendiente agendar llamada</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr"/>
@@ -1717,55 +1715,55 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="S20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
@@ -1774,10 +1772,10 @@
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1792,33 +1790,29 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
@@ -1846,61 +1840,61 @@
         <v>17</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G22" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I22" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="R22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="U22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="V22" s="4" t="n">
         <v>14</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>14</v>
@@ -1914,67 +1908,67 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="O23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="V23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2021,7 +2015,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-05-31</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2033,107 +2027,107 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2144,67 +2138,67 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>14</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -2214,64 +2208,64 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>23</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>19</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>18</v>
@@ -2284,52 +2278,52 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>6</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>2</v>
@@ -2338,7 +2332,7 @@
         <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2353,16 +2347,18 @@
           <t>Smart Duck</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="E7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>1</v>
@@ -2400,10 +2396,10 @@
       <c r="R7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2418,64 +2414,64 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="F8" s="4" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="4" t="n">
+      <c r="S8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>10</v>
@@ -2488,13 +2484,13 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>1</v>
@@ -2503,18 +2499,18 @@
         <v>1</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2531,7 +2527,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
@@ -2543,10 +2539,10 @@
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -2556,49 +2552,49 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
@@ -2607,13 +2603,13 @@
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>8</v>
@@ -2626,67 +2622,67 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="P11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -2696,67 +2692,67 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-02)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-01</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -679,19 +679,19 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>6</v>
@@ -700,25 +700,25 @@
         <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,13 +754,13 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>14</v>
@@ -769,31 +769,31 @@
         <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>7</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>17</v>
@@ -900,34 +900,34 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="N7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="Q7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="U7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>9</v>
@@ -959,47 +959,47 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1032,49 +1032,49 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="M9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1107,49 +1107,49 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1182,19 +1182,19 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>10</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>6</v>
@@ -1215,16 +1215,16 @@
         <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1257,49 +1257,49 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1332,28 +1332,28 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>3</v>
@@ -1362,19 +1362,19 @@
         <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1407,49 +1407,49 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1483,43 +1483,43 @@
         <v>22</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q15" s="6" t="n">
+      <c r="R15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>10</v>
@@ -1555,10 +1555,10 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
@@ -1608,7 +1608,9 @@
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
-      <c r="R17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1657,9 +1659,7 @@
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -1737,34 +1737,34 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
@@ -1773,7 +1773,7 @@
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>3</v>
@@ -1808,14 +1808,12 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
@@ -1826,7 +1824,9 @@
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
-      <c r="V21" s="6" t="inlineStr"/>
+      <c r="V21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="W21" s="6" t="n">
         <v>2</v>
       </c>
@@ -1864,43 +1864,43 @@
         <v>15</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="Q22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="T22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="U22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="V22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>17</v>
@@ -1932,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="O23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="P23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="V23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>103</v>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-01</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2162,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>27</v>
@@ -2232,46 +2232,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>24</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -2305,28 +2305,28 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>2</v>
@@ -2335,7 +2335,7 @@
         <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
@@ -2399,10 +2399,10 @@
       <c r="Q7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2441,43 +2441,43 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="n">
+      <c r="R8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>11</v>
@@ -2508,12 +2508,12 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
@@ -2542,7 +2542,7 @@
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>4</v>
@@ -2579,7 +2579,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>3</v>
@@ -2588,16 +2588,16 @@
         <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
@@ -2606,16 +2606,16 @@
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="T10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -2646,46 +2646,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>35</v>
@@ -2716,46 +2716,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>103</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-03)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-02</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -679,16 +679,16 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>6</v>
@@ -697,28 +697,28 @@
         <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>8</v>
@@ -754,10 +754,10 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>14</v>
@@ -766,34 +766,34 @@
         <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>8</v>
@@ -828,43 +828,43 @@
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="P6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>16</v>
@@ -900,35 +900,33 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="M7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="P7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="T7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="V7" s="6" t="n">
         <v>9</v>
       </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -957,47 +955,47 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1030,49 +1028,49 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1105,46 +1103,46 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="S10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>4</v>
@@ -1180,16 +1178,16 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>10</v>
@@ -1198,7 +1196,7 @@
         <v>10</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>6</v>
@@ -1210,16 +1208,16 @@
         <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>10</v>
@@ -1258,43 +1256,43 @@
         <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>2</v>
@@ -1330,46 +1328,46 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="J13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>1</v>
@@ -1405,43 +1403,43 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J14" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="U14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1478,46 +1476,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P15" s="6" t="n">
+      <c r="Q15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>15</v>
@@ -1552,10 +1550,10 @@
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
@@ -1605,7 +1603,9 @@
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
-      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1618,9 +1618,7 @@
       <c r="U17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1652,9 +1650,7 @@
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1736,28 +1732,28 @@
         <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>2</v>
@@ -1766,16 +1762,16 @@
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1806,9 +1802,7 @@
       <c r="I21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
@@ -1819,9 +1813,11 @@
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
-      <c r="U21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
@@ -1857,49 +1853,49 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="J22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="P22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="S22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="T22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="T22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="U22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
@@ -1928,49 +1924,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="N23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="T23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="O23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="U23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="V23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2017,7 +2013,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-02</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -2059,77 +2055,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -2161,43 +2157,43 @@
         <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>22</v>
@@ -2231,46 +2227,46 @@
         <v>24</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -2298,28 +2294,28 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>2</v>
@@ -2328,7 +2324,7 @@
         <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>3</v>
@@ -2337,7 +2333,7 @@
         <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2392,10 +2388,10 @@
       <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2434,43 +2430,43 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="n">
+      <c r="Q8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>11</v>
@@ -2503,10 +2499,10 @@
       <c r="G9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2523,7 +2519,7 @@
         <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
@@ -2535,7 +2531,7 @@
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>4</v>
@@ -2572,25 +2568,25 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
@@ -2599,16 +2595,16 @@
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="S10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2642,46 +2638,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="N11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>37</v>
@@ -2712,49 +2708,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="U12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-04)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-03</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -679,13 +679,13 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>6</v>
@@ -694,31 +694,31 @@
         <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,7 +754,7 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>14</v>
@@ -763,34 +763,34 @@
         <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>8</v>
@@ -825,43 +825,43 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="S6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>16</v>
@@ -900,33 +900,33 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="U7" s="6" t="inlineStr"/>
+      <c r="V7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="n">
         <v>4</v>
       </c>
@@ -959,42 +959,42 @@
       <c r="I8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>12</v>
@@ -1030,43 +1030,43 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -1105,46 +1105,46 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="Q10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1183,10 +1183,10 @@
         <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>10</v>
@@ -1195,7 +1195,7 @@
         <v>10</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>6</v>
@@ -1207,19 +1207,19 @@
         <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>8</v>
@@ -1255,49 +1255,49 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="L12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="O12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="P12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1330,22 +1330,22 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>3</v>
@@ -1354,25 +1354,25 @@
         <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1405,40 +1405,40 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>2</v>
@@ -1478,43 +1478,43 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O15" s="6" t="n">
+      <c r="P15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>15</v>
@@ -1551,10 +1551,10 @@
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1604,7 +1604,9 @@
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1617,10 +1619,10 @@
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1651,9 +1653,7 @@
       <c r="I18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
@@ -1733,28 +1733,28 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="L20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>2</v>
@@ -1763,13 +1763,13 @@
         <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1803,9 +1803,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
@@ -1816,9 +1814,11 @@
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
-      <c r="T21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
@@ -1857,46 +1857,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="M22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="R22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="S22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="T22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>21</v>
@@ -1928,46 +1928,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="M23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="N23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="T23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>105</v>
@@ -2017,7 +2017,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-03</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2059,77 +2059,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -2158,46 +2158,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>26</v>
@@ -2228,46 +2228,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>20</v>
@@ -2298,46 +2298,46 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2389,10 +2389,10 @@
       <c r="O7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -2434,46 +2434,46 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="n">
+      <c r="P8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>12</v>
@@ -2503,7 +2503,9 @@
       <c r="G9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2520,7 +2522,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
@@ -2532,7 +2534,7 @@
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>4</v>
@@ -2541,7 +2543,7 @@
         <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2578,16 +2580,16 @@
         <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
@@ -2596,22 +2598,22 @@
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="R10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2642,46 +2644,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>34</v>
@@ -2712,46 +2714,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>105</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-05)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-04</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>8</v>
@@ -760,34 +760,34 @@
         <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>8</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="N6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="R6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>13</v>
@@ -899,33 +899,33 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="K7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="N7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="R7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="T7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>8</v>
@@ -956,45 +956,45 @@
       <c r="H8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>11</v>
@@ -1030,46 +1030,46 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>1</v>
@@ -1105,46 +1105,46 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="P10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>6</v>
@@ -1180,10 +1180,10 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>10</v>
@@ -1192,7 +1192,7 @@
         <v>10</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6</v>
@@ -1204,22 +1204,22 @@
         <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1258,43 +1258,43 @@
         <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="N12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="O12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>1</v>
@@ -1330,19 +1330,19 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3</v>
@@ -1351,25 +1351,25 @@
         <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>1</v>
@@ -1405,37 +1405,37 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="S14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>2</v>
@@ -1478,46 +1478,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N15" s="6" t="n">
+      <c r="O15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>19</v>
@@ -1550,10 +1550,10 @@
         <v>1</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
@@ -1603,7 +1603,9 @@
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1616,10 +1618,10 @@
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1650,9 +1652,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
@@ -1733,25 +1733,25 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
@@ -1760,19 +1760,19 @@
         <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
@@ -1813,9 +1813,11 @@
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="T21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>1</v>
@@ -1857,46 +1859,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="J22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="L22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="Q22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="R22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="S22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>19</v>
@@ -1928,46 +1930,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="R23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="M23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="S23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>107</v>
@@ -2017,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-04</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -2059,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -2158,46 +2160,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>25</v>
@@ -2228,43 +2230,43 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>20</v>
@@ -2298,43 +2300,43 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>2</v>
@@ -2386,10 +2388,10 @@
       <c r="N7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2400,7 +2402,7 @@
         <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>2</v>
@@ -2434,43 +2436,43 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
+      <c r="O8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>12</v>
@@ -2519,7 +2521,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
@@ -2531,7 +2533,7 @@
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>4</v>
@@ -2540,7 +2542,7 @@
         <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2577,40 +2579,40 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>6</v>
@@ -2644,46 +2646,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>37</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>34</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>37</v>
@@ -2714,46 +2716,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="R12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>107</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-06)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-05</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-05</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-07)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-06</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-06</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-08)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-07</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="U4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>6</v>
@@ -757,34 +757,34 @@
         <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>8</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="M6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>11</v>
@@ -900,36 +900,36 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="J7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="M7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="Q7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="S7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="W7" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -956,48 +956,50 @@
       <c r="H8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -1030,49 +1032,49 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1105,43 +1107,43 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="O10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -1180,7 +1182,7 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>10</v>
@@ -1189,7 +1191,7 @@
         <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>6</v>
@@ -1201,28 +1203,28 @@
         <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1255,47 +1257,45 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="M12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="N12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V12" s="4" t="inlineStr"/>
       <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1328,16 +1328,16 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>3</v>
@@ -1346,25 +1346,25 @@
         <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>1</v>
@@ -1403,34 +1403,34 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>2</v>
@@ -1445,7 +1445,7 @@
         <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1476,49 +1476,49 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M15" s="6" t="n">
+      <c r="N15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="W15" s="6" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -1548,9 +1548,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
@@ -1600,7 +1598,9 @@
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1613,16 +1613,14 @@
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1661,7 +1659,9 @@
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1731,22 +1731,22 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="L20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
@@ -1755,19 +1755,19 @@
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
@@ -1810,9 +1810,11 @@
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="S21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>1</v>
@@ -1821,10 +1823,10 @@
         <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1857,46 +1859,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="P22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="Q22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="R22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>12</v>
@@ -1928,49 +1930,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="R23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2017,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-07</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -2059,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -2161,43 +2163,43 @@
         <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>24</v>
@@ -2228,49 +2230,49 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2298,40 +2300,40 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>2</v>
@@ -2383,10 +2385,10 @@
       <c r="M7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2397,13 +2399,13 @@
         <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>1</v>
@@ -2434,40 +2436,40 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>12</v>
@@ -2516,7 +2518,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
@@ -2528,7 +2530,7 @@
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>4</v>
@@ -2537,16 +2539,16 @@
         <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2574,40 +2576,40 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>6</v>
@@ -2644,49 +2646,49 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="T11" s="10" t="n">
+      <c r="U11" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="U11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="V11" s="10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -2714,49 +2716,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-09)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-08</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -685,40 +685,40 @@
         <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>9</v>
@@ -754,34 +754,34 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>8</v>
@@ -793,7 +793,7 @@
         <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>11</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="L6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>8</v>
@@ -899,39 +899,39 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="I7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="L7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="P7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="R7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="T7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="U7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W7" s="6" t="n">
-        <v>4</v>
-      </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -962,46 +962,46 @@
         <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>11</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1034,48 +1034,48 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W9" s="6" t="inlineStr"/>
+      <c r="V9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1107,46 +1107,46 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="N10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>4</v>
@@ -1188,7 +1188,7 @@
         <v>10</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>6</v>
@@ -1200,28 +1200,28 @@
         <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>11</v>
@@ -1257,47 +1257,47 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="L12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1333,10 +1333,10 @@
         <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>3</v>
@@ -1345,25 +1345,25 @@
         <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>1</v>
@@ -1405,49 +1405,49 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W14" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W14" s="4" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1478,46 +1478,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L15" s="6" t="n">
+      <c r="M15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>16</v>
@@ -1599,7 +1599,9 @@
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1612,16 +1614,14 @@
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
@@ -1660,10 +1660,10 @@
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1731,46 +1731,46 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="K20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V20" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>4</v>
@@ -1809,9 +1809,11 @@
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>1</v>
@@ -1820,10 +1822,10 @@
         <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>2</v>
@@ -1859,43 +1861,43 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="P22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="Q22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>12</v>
@@ -1930,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="P23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="Q23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>96</v>
@@ -2019,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-08</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -2061,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -2160,46 +2162,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>23</v>
@@ -2230,46 +2232,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2303,34 +2305,34 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>2</v>
@@ -2339,7 +2341,7 @@
         <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>3</v>
@@ -2382,10 +2384,10 @@
       <c r="L7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2396,13 +2398,13 @@
         <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>1</v>
@@ -2439,34 +2441,34 @@
         <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>12</v>
@@ -2475,7 +2477,7 @@
         <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>15</v>
@@ -2515,7 +2517,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
@@ -2527,7 +2529,7 @@
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>4</v>
@@ -2536,16 +2538,16 @@
         <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
@@ -2579,34 +2581,34 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>6</v>
@@ -2646,46 +2648,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="J11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="S11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="T11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="U11" s="10" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>32</v>
@@ -2716,46 +2718,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>96</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-10)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-09</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,31 +754,31 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>8</v>
@@ -790,7 +790,7 @@
         <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -825,43 +825,43 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>8</v>
@@ -899,37 +899,37 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="K7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="O7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="S7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>1</v>
@@ -961,43 +961,43 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>8</v>
@@ -1039,42 +1039,42 @@
         <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="inlineStr"/>
+      <c r="V9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="W9" s="6" t="n">
         <v>3</v>
       </c>
@@ -1109,46 +1109,46 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="R10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="S10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>3</v>
@@ -1187,7 +1187,7 @@
         <v>10</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>6</v>
@@ -1199,28 +1199,28 @@
         <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>11</v>
@@ -1259,42 +1259,42 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="V12" s="4" t="n">
         <v>3</v>
       </c>
@@ -1332,10 +1332,10 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>3</v>
@@ -1344,25 +1344,25 @@
         <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>1</v>
@@ -1407,28 +1407,28 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>2</v>
@@ -1443,10 +1443,10 @@
         <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>2</v>
@@ -1480,46 +1480,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K15" s="6" t="n">
+      <c r="L15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>18</v>
@@ -1600,7 +1600,9 @@
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1613,16 +1615,14 @@
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
@@ -1661,10 +1661,10 @@
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
     </row>
@@ -1733,46 +1733,46 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="V20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2</v>
@@ -1810,9 +1810,11 @@
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="Q21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>1</v>
@@ -1821,14 +1823,12 @@
         <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V21" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1861,46 +1861,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="N22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="O22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="P22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>17</v>
@@ -1932,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="O23" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="P23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>95</v>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-09</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2162,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>22</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>19</v>
@@ -2232,46 +2232,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -2302,34 +2302,34 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>2</v>
@@ -2338,7 +2338,7 @@
         <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2381,10 +2381,10 @@
       <c r="K7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2395,13 +2395,13 @@
         <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>1</v>
@@ -2438,34 +2438,34 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>12</v>
@@ -2474,7 +2474,7 @@
         <v>12</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>15</v>
@@ -2514,7 +2514,7 @@
         <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
@@ -2526,7 +2526,7 @@
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>4</v>
@@ -2535,16 +2535,16 @@
         <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
@@ -2578,34 +2578,34 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
@@ -2617,7 +2617,7 @@
         <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>7</v>
@@ -2648,46 +2648,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="R11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="S11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="T11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>35</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>33</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>35</v>
@@ -2718,46 +2718,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>85</v>
-      </c>
       <c r="O12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>95</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-11)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-10</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>8</v>
@@ -754,28 +754,28 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>8</v>
@@ -787,13 +787,13 @@
         <v>8</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>10</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>10</v>
@@ -900,36 +900,38 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="J7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="R7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>2</v>
@@ -961,46 +963,46 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>4</v>
@@ -1036,42 +1038,42 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
       </c>
@@ -1112,43 +1114,43 @@
         <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="Q10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="R10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>1</v>
@@ -1184,7 +1186,7 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>6</v>
@@ -1196,28 +1198,28 @@
         <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>11</v>
@@ -1259,44 +1261,44 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="U12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>2</v>
@@ -1332,7 +1334,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>3</v>
@@ -1341,25 +1343,25 @@
         <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>1</v>
@@ -1371,7 +1373,7 @@
         <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>7</v>
@@ -1407,25 +1409,25 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>2</v>
@@ -1440,13 +1442,13 @@
         <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>1</v>
@@ -1480,46 +1482,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="R15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>15</v>
@@ -1599,7 +1601,9 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1612,16 +1616,14 @@
       <c r="O17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
@@ -1660,10 +1662,10 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
@@ -1733,47 +1735,45 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1807,9 +1807,11 @@
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="P21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
@@ -1818,15 +1820,15 @@
         <v>1</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V21" s="6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="U21" s="6" t="inlineStr"/>
+      <c r="V21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1861,43 +1863,43 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="M22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="N22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="O22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>17</v>
@@ -1932,46 +1934,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>92</v>
@@ -2021,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-10</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2164,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>20</v>
@@ -2232,46 +2234,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2302,10 +2304,10 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>2</v>
@@ -2314,7 +2316,7 @@
         <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>3</v>
@@ -2323,10 +2325,10 @@
         <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>2</v>
@@ -2335,7 +2337,7 @@
         <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
@@ -2378,10 +2380,10 @@
       <c r="J7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2392,13 +2394,13 @@
         <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>1</v>
@@ -2438,31 +2440,31 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>12</v>
@@ -2471,13 +2473,13 @@
         <v>12</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>13</v>
@@ -2511,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
@@ -2523,7 +2525,7 @@
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>4</v>
@@ -2532,23 +2534,21 @@
         <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2576,31 +2576,31 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
@@ -2612,10 +2612,10 @@
         <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2646,46 +2646,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>30</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="Q11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="S11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="T11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="U11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>34</v>
@@ -2716,46 +2716,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>92</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-12)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-11</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="S4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,25 +754,25 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>8</v>
@@ -784,16 +784,16 @@
         <v>8</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>13</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>5</v>
@@ -899,39 +899,41 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="I7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="Q7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="T7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>2</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>4</v>
@@ -963,49 +965,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1038,44 +1040,44 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>1</v>
@@ -1111,48 +1113,48 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1193,28 +1195,28 @@
         <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>11</v>
@@ -1223,7 +1225,7 @@
         <v>11</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>10</v>
@@ -1259,44 +1261,44 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="T12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>3</v>
@@ -1338,25 +1340,25 @@
         <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>1</v>
@@ -1368,10 +1370,10 @@
         <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>8</v>
@@ -1407,22 +1409,22 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>2</v>
@@ -1437,13 +1439,13 @@
         <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1480,46 +1482,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>13</v>
@@ -1598,7 +1600,9 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1611,16 +1615,14 @@
       <c r="N17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
@@ -1659,10 +1661,10 @@
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1733,10 +1735,10 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>2</v>
@@ -1745,33 +1747,33 @@
         <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="U20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1806,9 +1808,11 @@
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr"/>
+      <c r="N21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="O21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>1</v>
@@ -1817,18 +1821,16 @@
         <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U21" s="6" t="inlineStr"/>
-      <c r="V21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="T21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1861,46 +1863,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="L22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="M22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="N22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="S22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>22</v>
@@ -1932,46 +1934,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>92</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>95</v>
@@ -2021,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-11</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2164,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="R4" s="4" t="n">
+      <c r="T4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>23</v>
@@ -2232,43 +2234,43 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>15</v>
@@ -2302,7 +2304,7 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>2</v>
@@ -2311,7 +2313,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>3</v>
@@ -2320,28 +2322,28 @@
         <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2375,10 +2377,10 @@
       <c r="I7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2389,13 +2391,13 @@
         <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>1</v>
@@ -2438,28 +2440,28 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>12</v>
@@ -2468,16 +2470,16 @@
         <v>12</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>11</v>
@@ -2508,7 +2510,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>3</v>
@@ -2520,7 +2522,7 @@
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>4</v>
@@ -2529,23 +2531,21 @@
         <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
     </row>
@@ -2580,22 +2580,22 @@
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
@@ -2607,13 +2607,13 @@
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="T10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -2647,43 +2647,43 @@
         <v>30</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="P11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="R11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="S11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>36</v>
@@ -2714,46 +2714,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>92</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>95</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-13)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-12</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-12</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-14)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-13</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-13</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-15)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-14</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="R4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="V4" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>8</v>
@@ -757,19 +757,19 @@
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>8</v>
@@ -781,19 +781,19 @@
         <v>8</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>11</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>11</v>
@@ -899,41 +899,41 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="P7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="S7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>2</v>
@@ -965,49 +965,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1040,44 +1040,44 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>2</v>
@@ -1113,47 +1113,47 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U10" s="4" t="inlineStr"/>
+      <c r="V10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1192,28 +1192,28 @@
         <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>11</v>
@@ -1222,10 +1222,10 @@
         <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>9</v>
@@ -1261,44 +1261,44 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="S12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>1</v>
@@ -1337,46 +1337,46 @@
         <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="M13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="V13" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1412,16 +1412,16 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>2</v>
@@ -1436,22 +1436,22 @@
         <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1482,46 +1482,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="T15" s="6" t="n">
+      <c r="U15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>18</v>
@@ -1599,7 +1599,9 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1612,16 +1614,14 @@
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
@@ -1660,10 +1660,10 @@
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
@@ -1735,7 +1735,7 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
@@ -1744,35 +1744,35 @@
         <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="T20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2</v>
@@ -1807,9 +1807,11 @@
       <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="N21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>1</v>
@@ -1818,18 +1820,16 @@
         <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T21" s="6" t="inlineStr"/>
-      <c r="U21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="S21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
     </row>
@@ -1863,46 +1863,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="L22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="M22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>23</v>
@@ -1934,46 +1934,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="O23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>101</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>101</v>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-14</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2065,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2164,43 +2164,43 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q4" s="4" t="n">
+      <c r="S4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>23</v>
@@ -2234,46 +2234,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>18</v>
@@ -2310,7 +2310,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>3</v>
@@ -2319,31 +2319,31 @@
         <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>7</v>
@@ -2374,10 +2374,10 @@
       <c r="H7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2388,13 +2388,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>1</v>
@@ -2440,25 +2440,25 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>12</v>
@@ -2467,16 +2467,16 @@
         <v>12</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>11</v>
@@ -2519,7 +2519,7 @@
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>4</v>
@@ -2528,23 +2528,21 @@
         <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
@@ -2577,22 +2575,22 @@
         <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="L10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
@@ -2604,13 +2602,13 @@
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="S10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2644,43 +2642,43 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="O11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="Q11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>36</v>
@@ -2714,46 +2712,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>101</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>101</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-16)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-15</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="T4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>4</v>
@@ -754,19 +754,19 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>8</v>
@@ -778,22 +778,22 @@
         <v>8</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="U5" s="6" t="n">
+      <c r="V5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>13</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>15</v>
@@ -900,37 +900,39 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="O7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="R7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -965,49 +967,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="U8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="W8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1040,47 +1042,47 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1113,44 +1115,44 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="4" t="inlineStr"/>
+      <c r="U10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="4" t="inlineStr"/>
-      <c r="V10" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>4</v>
@@ -1189,28 +1191,28 @@
         <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>11</v>
@@ -1219,13 +1221,13 @@
         <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1261,47 +1263,47 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="R12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1334,48 +1336,48 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="L13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="W13" s="6" t="inlineStr"/>
+      <c r="V13" s="6" t="inlineStr"/>
+      <c r="W13" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1407,16 +1409,16 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>2</v>
@@ -1431,22 +1433,22 @@
         <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>1</v>
@@ -1480,46 +1482,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="T15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>19</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>19</v>
@@ -1609,16 +1611,14 @@
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
@@ -1657,10 +1657,10 @@
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
@@ -1739,38 +1739,38 @@
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>7</v>
@@ -1804,9 +1804,11 @@
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="M21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
@@ -1815,18 +1817,16 @@
         <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S21" s="6" t="inlineStr"/>
-      <c r="T21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="R21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
@@ -1864,43 +1864,43 @@
         <v>14</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="L22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="S22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>25</v>
@@ -1932,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="O23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>95</v>
-      </c>
       <c r="V23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>106</v>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-15</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2162,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="R4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>29</v>
@@ -2235,43 +2235,43 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>21</v>
@@ -2305,7 +2305,7 @@
         <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -2314,31 +2314,31 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>7</v>
@@ -2369,10 +2369,10 @@
       <c r="G7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2383,13 +2383,13 @@
         <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>1</v>
@@ -2438,22 +2438,22 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>12</v>
@@ -2462,22 +2462,22 @@
         <v>12</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>9</v>
@@ -2514,7 +2514,7 @@
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>4</v>
@@ -2523,23 +2523,21 @@
         <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
@@ -2570,22 +2568,22 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
@@ -2597,19 +2595,19 @@
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2640,46 +2638,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="N11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="P11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="R11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>33</v>
@@ -2710,46 +2708,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>95</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>106</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-17)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-16</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="P4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>2</v>
@@ -754,16 +754,16 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>8</v>
@@ -775,25 +775,25 @@
         <v>8</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="U5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>16</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>16</v>
@@ -899,37 +899,39 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="L7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="N7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="Q7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>2</v>
@@ -967,49 +969,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1042,47 +1044,47 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1115,47 +1117,47 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="4" t="inlineStr"/>
-      <c r="U10" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1188,28 +1190,28 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>11</v>
@@ -1218,16 +1220,16 @@
         <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>6</v>
@@ -1263,44 +1265,44 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="Q12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>2</v>
@@ -1336,44 +1338,42 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="K13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>4</v>
-      </c>
+      <c r="U13" s="6" t="inlineStr"/>
       <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="6" t="inlineStr"/>
     </row>
@@ -1410,10 +1410,10 @@
         <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
@@ -1428,22 +1428,22 @@
         <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1480,46 +1480,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="S15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>22</v>
@@ -1606,16 +1606,14 @@
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
@@ -1654,10 +1652,10 @@
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
@@ -1734,41 +1732,41 @@
         <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V20" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>4</v>
@@ -1801,9 +1799,11 @@
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="L21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
@@ -1812,21 +1812,21 @@
         <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="Q21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
       <c r="U21" s="6" t="inlineStr"/>
-      <c r="V21" s="6" t="inlineStr"/>
+      <c r="V21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1861,46 +1861,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="J22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="J22" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="K22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>20</v>
@@ -1932,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="L23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>106</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>103</v>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-16</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -2165,43 +2165,43 @@
         <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>30</v>
@@ -2232,46 +2232,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>19</v>
-      </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>16</v>
@@ -2302,7 +2302,7 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>3</v>
@@ -2311,37 +2311,37 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>6</v>
@@ -2369,7 +2369,9 @@
       <c r="G7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2380,13 +2382,13 @@
         <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>1</v>
@@ -2441,16 +2443,16 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>12</v>
@@ -2459,22 +2461,22 @@
         <v>12</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>9</v>
@@ -2511,7 +2513,7 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>4</v>
@@ -2520,23 +2522,21 @@
         <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
@@ -2568,19 +2568,19 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="J10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>6</v>
@@ -2592,22 +2592,22 @@
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>7</v>
@@ -2638,46 +2638,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="M11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="O11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="Q11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>34</v>
@@ -2708,46 +2708,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>106</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>103</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-18)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-17</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -679,43 +679,43 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>2</v>
@@ -754,13 +754,13 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>8</v>
@@ -772,28 +772,28 @@
         <v>8</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="S5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>14</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>19</v>
@@ -900,35 +900,35 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="K7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>2</v>
@@ -936,9 +936,7 @@
       <c r="U7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="V7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -970,46 +968,46 @@
         <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1042,46 +1040,46 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="W9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="V9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1116,41 +1114,41 @@
         <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1186,25 +1184,25 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>11</v>
@@ -1213,19 +1211,19 @@
         <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>8</v>
@@ -1261,47 +1259,47 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="P12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1334,19 +1332,19 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>1</v>
@@ -1358,21 +1356,21 @@
         <v>1</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="T13" s="6" t="inlineStr"/>
       <c r="U13" s="6" t="inlineStr"/>
-      <c r="V13" s="6" t="inlineStr"/>
+      <c r="V13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1405,10 +1403,10 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
@@ -1423,22 +1421,22 @@
         <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>1</v>
@@ -1481,43 +1479,43 @@
         <v>11</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="R15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>4</v>
@@ -1564,7 +1562,9 @@
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
-      <c r="W16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1601,16 +1601,14 @@
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
@@ -1649,10 +1647,10 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
@@ -1727,44 +1725,44 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2</v>
@@ -1796,9 +1794,11 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="K21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
@@ -1807,21 +1807,21 @@
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="P21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
-      <c r="U21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1859,46 +1859,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="S22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V22" s="4" t="n">
         <v>22</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>22</v>
@@ -1930,49 +1930,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R23" s="8" t="n">
+      <c r="V23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>92</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>106</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2019,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-17</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2061,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -2160,46 +2160,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="P4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>26</v>
@@ -2230,43 +2230,43 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
@@ -2306,10 +2306,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>2</v>
@@ -2318,7 +2318,7 @@
         <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>3</v>
@@ -2327,19 +2327,19 @@
         <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>5</v>
@@ -2377,13 +2377,13 @@
         <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>1</v>
@@ -2438,16 +2438,16 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>12</v>
@@ -2456,28 +2456,28 @@
         <v>12</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>8</v>
@@ -2508,7 +2508,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>4</v>
@@ -2517,23 +2517,21 @@
         <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
@@ -2566,16 +2564,16 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>6</v>
@@ -2587,22 +2585,22 @@
         <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>7</v>
@@ -2636,49 +2634,49 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="L11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="N11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="P11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -2706,49 +2704,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q12" s="8" t="n">
+      <c r="U12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>92</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>106</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-19)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-18</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="N4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>4</v>
@@ -754,10 +754,10 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>8</v>
@@ -769,28 +769,28 @@
         <v>8</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="R5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="T6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>15</v>
@@ -900,32 +900,32 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="J7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>2</v>
@@ -933,10 +933,10 @@
       <c r="T7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="U7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="inlineStr"/>
+      <c r="V7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="W7" s="6" t="n">
         <v>3</v>
       </c>
@@ -967,46 +967,46 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>4</v>
@@ -1042,43 +1042,43 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="U9" s="6" t="inlineStr"/>
+      <c r="V9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W9" s="6" t="n">
         <v>1</v>
       </c>
@@ -1113,44 +1113,44 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q10" s="4" t="inlineStr"/>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>3</v>
@@ -1189,19 +1189,19 @@
         <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>11</v>
@@ -1210,19 +1210,19 @@
         <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>8</v>
@@ -1261,44 +1261,44 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="O12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>6</v>
@@ -1334,16 +1334,16 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>1</v>
@@ -1355,19 +1355,19 @@
         <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="S13" s="6" t="inlineStr"/>
       <c r="T13" s="6" t="inlineStr"/>
-      <c r="U13" s="6" t="inlineStr"/>
+      <c r="U13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="V13" s="6" t="n">
         <v>2</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
@@ -1420,22 +1420,22 @@
         <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>1</v>
@@ -1478,46 +1478,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="Q15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>6</v>
@@ -1563,7 +1563,9 @@
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="inlineStr"/>
+      <c r="V16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1600,16 +1602,14 @@
       <c r="I17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
@@ -1648,10 +1648,10 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -1730,38 +1730,38 @@
         <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1795,9 +1795,11 @@
       </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="J21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
@@ -1806,26 +1808,26 @@
         <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
-      <c r="T21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>2</v>
@@ -1861,46 +1863,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="R22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="S22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>20</v>
-      </c>
       <c r="V22" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>19</v>
@@ -1932,43 +1934,43 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="T23" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="U23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>91</v>
@@ -2021,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-18</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
@@ -2162,46 +2164,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>27</v>
@@ -2232,46 +2234,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -2305,10 +2307,10 @@
         <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>2</v>
@@ -2317,7 +2319,7 @@
         <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>3</v>
@@ -2326,22 +2328,22 @@
         <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2376,13 +2378,13 @@
         <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>1</v>
@@ -2440,13 +2442,13 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>12</v>
@@ -2455,28 +2457,28 @@
         <v>12</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>8</v>
@@ -2516,23 +2518,21 @@
         <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
@@ -2566,13 +2566,13 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>6</v>
@@ -2584,22 +2584,22 @@
         <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>7</v>
@@ -2636,46 +2636,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="K11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="M11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>27</v>
@@ -2706,43 +2706,43 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>91</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-20)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-19</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-19</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-21)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-20</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-20</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-22)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-21</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="K4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="O4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="Q4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -754,7 +754,7 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>8</v>
@@ -766,34 +766,34 @@
         <v>8</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>17</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>17</v>
@@ -899,30 +899,30 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>2</v>
@@ -930,12 +930,12 @@
       <c r="S7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="V7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>1</v>
@@ -967,49 +967,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1042,45 +1042,45 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1113,47 +1113,47 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1186,19 +1186,19 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>11</v>
@@ -1207,19 +1207,19 @@
         <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>8</v>
@@ -1261,47 +1261,47 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="N12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1334,13 +1334,13 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>1</v>
@@ -1352,27 +1352,27 @@
         <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr"/>
       <c r="S13" s="6" t="inlineStr"/>
-      <c r="T13" s="6" t="inlineStr"/>
+      <c r="T13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="U13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1417,22 +1417,22 @@
         <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>1</v>
@@ -1478,46 +1478,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>15</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="P15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="S15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>11</v>
@@ -1562,9 +1562,11 @@
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>2</v>
@@ -1599,16 +1601,14 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
@@ -1647,10 +1647,10 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
@@ -1727,38 +1727,38 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
@@ -1767,7 +1767,7 @@
         <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1796,7 +1796,7 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
@@ -1805,29 +1805,29 @@
         <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="N21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
@@ -1863,46 +1863,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="P22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="V22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>17</v>
@@ -1934,46 +1934,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="T23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="U23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>94</v>
@@ -2023,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-21</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2065,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2164,46 +2164,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>26</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>27</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>26</v>
@@ -2237,43 +2237,43 @@
         <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2304,10 +2304,10 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>2</v>
@@ -2316,7 +2316,7 @@
         <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>3</v>
@@ -2325,22 +2325,22 @@
         <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2375,13 +2375,13 @@
         <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>1</v>
@@ -2411,7 +2411,7 @@
         <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -2445,7 +2445,7 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>12</v>
@@ -2454,28 +2454,28 @@
         <v>12</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>8</v>
@@ -2515,23 +2515,21 @@
         <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
@@ -2569,7 +2567,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>6</v>
@@ -2581,22 +2579,22 @@
         <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="N10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>7</v>
@@ -2605,7 +2603,7 @@
         <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2636,46 +2634,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>37</v>
-      </c>
       <c r="J11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="L11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="N11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>33</v>
@@ -2706,46 +2704,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>94</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-23)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-22</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -679,43 +679,43 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="N4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -763,37 +763,37 @@
         <v>8</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>18</v>
@@ -828,43 +828,43 @@
         <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="S6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>13</v>
@@ -899,27 +899,29 @@
       <c r="H7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="J7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="M7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>2</v>
@@ -927,12 +929,12 @@
       <c r="R7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>1</v>
@@ -967,46 +969,46 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>3</v>
@@ -1045,39 +1047,39 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>1</v>
@@ -1113,41 +1115,41 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" s="4" t="inlineStr"/>
-      <c r="Q10" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>1</v>
@@ -1186,16 +1188,16 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>11</v>
@@ -1204,28 +1206,28 @@
         <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>8</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1264,44 +1266,44 @@
         <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="M12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1334,10 +1336,10 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>1</v>
@@ -1349,27 +1351,27 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q13" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="Q13" s="6" t="inlineStr"/>
       <c r="R13" s="6" t="inlineStr"/>
-      <c r="S13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="T13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>3</v>
@@ -1414,22 +1416,22 @@
         <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>1</v>
@@ -1444,10 +1446,10 @@
         <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1481,43 +1483,43 @@
         <v>15</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="O15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>8</v>
@@ -1561,9 +1563,11 @@
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
-      <c r="T16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V16" s="4" t="n">
         <v>2</v>
@@ -1601,13 +1605,13 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
@@ -1618,7 +1622,9 @@
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
-      <c r="V17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1648,10 +1654,10 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -1732,32 +1738,32 @@
         <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
@@ -1766,7 +1772,7 @@
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>5</v>
@@ -1804,33 +1810,31 @@
         <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="M21" s="6" t="inlineStr"/>
+      <c r="N21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1863,46 +1867,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="P22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="V22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>15</v>
@@ -1934,46 +1938,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P23" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>95</v>
-      </c>
       <c r="Q23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="T23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>93</v>
@@ -2023,7 +2027,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-22</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -2065,77 +2069,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -2164,46 +2168,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>27</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>26</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>27</v>
@@ -2234,46 +2238,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>20</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -2304,40 +2308,40 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
@@ -2372,13 +2376,13 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>1</v>
@@ -2408,7 +2412,7 @@
         <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>2</v>
@@ -2442,7 +2446,7 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>12</v>
@@ -2451,28 +2455,28 @@
         <v>12</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>8</v>
@@ -2481,7 +2485,7 @@
         <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
@@ -2512,23 +2516,21 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
@@ -2564,7 +2566,7 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>6</v>
@@ -2576,22 +2578,22 @@
         <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>7</v>
@@ -2600,7 +2602,7 @@
         <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>6</v>
@@ -2634,43 +2636,43 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="K11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>33</v>
@@ -2704,46 +2706,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="S12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>93</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-24)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-23</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -679,40 +679,40 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>5</v>
@@ -760,43 +760,43 @@
         <v>8</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -825,49 +825,49 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="T6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="U6" s="4" t="n">
+      <c r="W6" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -900,25 +900,25 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="L7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>2</v>
@@ -926,18 +926,18 @@
       <c r="Q7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>2</v>
@@ -969,49 +969,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="S8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1044,44 +1044,44 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="R9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W9" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1113,38 +1113,38 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>1</v>
@@ -1186,13 +1186,13 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>11</v>
@@ -1201,19 +1201,19 @@
         <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>8</v>
@@ -1222,7 +1222,7 @@
         <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
@@ -1261,47 +1261,47 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1334,7 +1334,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>1</v>
@@ -1346,30 +1346,30 @@
         <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P13" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="P13" s="6" t="inlineStr"/>
       <c r="Q13" s="6" t="inlineStr"/>
-      <c r="R13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="S13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>4</v>
@@ -1411,22 +1411,22 @@
         <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>1</v>
@@ -1441,13 +1441,13 @@
         <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1478,49 +1478,49 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="N15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="W15" s="6" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1560,15 +1560,17 @@
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>1</v>
@@ -1606,9 +1608,7 @@
       <c r="I17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
@@ -1619,10 +1619,10 @@
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
-      <c r="U17" s="6" t="inlineStr"/>
-      <c r="V17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1649,10 +1649,10 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1731,32 +1731,32 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
@@ -1765,13 +1765,13 @@
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1803,34 +1803,34 @@
         <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U21" s="6" t="inlineStr"/>
+      <c r="V21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1865,46 +1865,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="N22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="O22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="U22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>13</v>
@@ -1936,49 +1936,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="N23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="N23" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="O23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="S23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2025,7 +2025,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-23</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -2067,77 +2067,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -2166,46 +2166,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>21</v>
@@ -2239,43 +2239,43 @@
         <v>20</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2312,7 +2312,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>3</v>
@@ -2321,22 +2321,22 @@
         <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
@@ -2345,7 +2345,7 @@
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>3</v>
@@ -2377,7 +2377,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
@@ -2407,7 +2407,7 @@
         <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>2</v>
@@ -2450,28 +2450,28 @@
         <v>12</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>8</v>
@@ -2480,13 +2480,13 @@
         <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="U8" s="4" t="n">
+      <c r="V8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -2517,17 +2517,15 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
@@ -2573,22 +2571,22 @@
         <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>7</v>
@@ -2597,13 +2595,13 @@
         <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -2634,49 +2632,49 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>38</v>
-      </c>
       <c r="J11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -2704,49 +2702,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="N12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-25)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-24</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -679,37 +679,37 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>5</v>
@@ -718,7 +718,7 @@
         <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>3</v>
@@ -757,43 +757,43 @@
         <v>8</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>14</v>
@@ -825,43 +825,43 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="S6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>16</v>
@@ -900,22 +900,22 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>2</v>
@@ -923,21 +923,21 @@
       <c r="P7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>4</v>
@@ -969,46 +969,46 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>2</v>
@@ -1046,38 +1046,36 @@
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="6" t="inlineStr"/>
     </row>
@@ -1114,32 +1112,32 @@
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>1</v>
@@ -1187,7 +1185,7 @@
         <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>11</v>
@@ -1196,19 +1194,19 @@
         <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>8</v>
@@ -1217,13 +1215,13 @@
         <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>6</v>
@@ -1258,45 +1256,45 @@
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="K12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>4</v>
@@ -1341,30 +1339,30 @@
         <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="6" t="inlineStr"/>
-      <c r="Q13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
@@ -1406,22 +1404,22 @@
         <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1</v>
@@ -1436,13 +1434,13 @@
         <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>2</v>
@@ -1476,46 +1474,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="P15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="U15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>8</v>
@@ -1557,15 +1555,17 @@
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
-      <c r="R16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V16" s="4" t="n">
         <v>1</v>
@@ -1603,9 +1603,7 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1616,10 +1614,10 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
-      <c r="T17" s="6" t="inlineStr"/>
-      <c r="U17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
@@ -1646,10 +1644,10 @@
       </c>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
@@ -1732,26 +1730,26 @@
         <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>2</v>
@@ -1760,10 +1758,10 @@
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1798,34 +1796,34 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U21" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1863,46 +1861,46 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="M22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="N22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="T22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>14</v>
@@ -1934,46 +1932,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="M23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="M23" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="N23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="R23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>82</v>
@@ -2023,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-24</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2065,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2164,43 +2162,43 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>21</v>
@@ -2234,46 +2232,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -2307,7 +2305,7 @@
         <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -2316,22 +2314,22 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
@@ -2340,7 +2338,7 @@
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2372,7 +2370,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>1</v>
@@ -2402,7 +2400,7 @@
         <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>2</v>
@@ -2445,28 +2443,28 @@
         <v>12</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>8</v>
@@ -2475,10 +2473,10 @@
         <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>8</v>
@@ -2512,17 +2510,15 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
@@ -2566,22 +2562,22 @@
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>7</v>
@@ -2590,13 +2586,13 @@
         <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2630,46 +2626,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>29</v>
@@ -2700,46 +2696,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="M12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>82</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-26)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-25</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -679,34 +679,34 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>5</v>
@@ -715,13 +715,13 @@
         <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="V4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="W4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -754,49 +754,49 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="V5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="W5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="W5" s="6" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -825,49 +825,49 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="R6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -900,19 +900,19 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>2</v>
@@ -920,28 +920,26 @@
       <c r="O7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="W7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -969,49 +967,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1043,41 +1041,41 @@
       <c r="H9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
-      <c r="W9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1109,32 +1107,32 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>1</v>
@@ -1182,7 +1180,7 @@
         <v>9</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>11</v>
@@ -1191,19 +1189,19 @@
         <v>11</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>8</v>
@@ -1212,13 +1210,13 @@
         <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>6</v>
@@ -1256,45 +1254,47 @@
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="J12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>1</v>
@@ -1336,30 +1336,30 @@
         <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="N13" s="6" t="inlineStr"/>
       <c r="O13" s="6" t="inlineStr"/>
-      <c r="P13" s="6" t="inlineStr"/>
+      <c r="P13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="Q13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>4</v>
@@ -1368,7 +1368,7 @@
         <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1401,22 +1401,22 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>1</v>
@@ -1431,19 +1431,19 @@
         <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1474,46 +1474,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="N15" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="T15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="U15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>10</v>
@@ -1554,15 +1554,17 @@
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U16" s="4" t="n">
         <v>1</v>
@@ -1613,10 +1615,10 @@
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
-      <c r="S17" s="6" t="inlineStr"/>
-      <c r="T17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
@@ -1644,9 +1646,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
@@ -1727,26 +1727,26 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>2</v>
@@ -1755,10 +1755,10 @@
         <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
@@ -1796,36 +1796,36 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>2</v>
@@ -1864,46 +1864,46 @@
         <v>12</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="L22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="M22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="S22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1932,49 +1932,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="L23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="M23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="Q23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="U23" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="V23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>81</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>82</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-25</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2063,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -2162,49 +2162,49 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="S4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -2232,49 +2232,49 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="S5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -2302,7 +2302,7 @@
         <v>3</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>3</v>
@@ -2311,22 +2311,22 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
@@ -2335,7 +2335,7 @@
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
@@ -2397,7 +2397,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>2</v>
@@ -2409,7 +2409,7 @@
         <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>1</v>
@@ -2440,28 +2440,28 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>15</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>8</v>
@@ -2470,19 +2470,19 @@
         <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -2510,14 +2510,12 @@
         <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
@@ -2559,22 +2557,22 @@
         <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>7</v>
@@ -2583,13 +2581,13 @@
         <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
@@ -2626,46 +2624,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>33</v>
-      </c>
       <c r="J11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>29</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>33</v>
@@ -2696,49 +2694,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="K12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="L12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="P12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="T12" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>81</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>82</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-27)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-26</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-27</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-26</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-28)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-27</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-28</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-27</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-29)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-28</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -679,31 +679,31 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>5</v>
@@ -712,13 +712,13 @@
         <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="U4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>3</v>
@@ -757,43 +757,43 @@
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>16</v>
@@ -828,43 +828,43 @@
         <v>8</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>15</v>
@@ -900,16 +900,16 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>2</v>
@@ -917,28 +917,26 @@
       <c r="N7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="V7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -970,43 +968,43 @@
         <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>2</v>
@@ -1041,35 +1039,35 @@
       <c r="H9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
@@ -1105,29 +1103,29 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>1</v>
@@ -1142,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>3</v>
@@ -1184,19 +1182,19 @@
         <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>8</v>
@@ -1205,19 +1203,19 @@
         <v>8</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>8</v>
@@ -1256,43 +1254,43 @@
         <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>2</v>
@@ -1331,30 +1329,30 @@
         <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="M13" s="6" t="inlineStr"/>
       <c r="N13" s="6" t="inlineStr"/>
-      <c r="O13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="P13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>4</v>
@@ -1363,7 +1361,7 @@
         <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>2</v>
@@ -1399,19 +1397,19 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
@@ -1426,16 +1424,16 @@
         <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1472,43 +1470,43 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="M15" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="T15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>10</v>
@@ -1551,15 +1549,17 @@
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>1</v>
@@ -1612,13 +1612,15 @@
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
-      <c r="R17" s="6" t="inlineStr"/>
-      <c r="S17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
-      <c r="V17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1727,23 +1729,23 @@
         <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
@@ -1752,10 +1754,10 @@
         <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
@@ -1764,7 +1766,7 @@
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>3</v>
@@ -1795,37 +1797,37 @@
       </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr"/>
+      <c r="N21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S21" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
@@ -1861,49 +1863,49 @@
         <v>14</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="K22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="L22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="R22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -1932,49 +1934,49 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="K23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="L23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="P23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="V23" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>80</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2021,7 +2023,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-28</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -2063,77 +2065,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -2162,49 +2164,49 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="R4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -2232,46 +2234,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>10</v>
@@ -2308,22 +2310,22 @@
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
@@ -2332,7 +2334,7 @@
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>3</v>
@@ -2341,7 +2343,7 @@
         <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2394,7 +2396,7 @@
         <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>2</v>
@@ -2406,7 +2408,7 @@
         <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>1</v>
@@ -2443,22 +2445,22 @@
         <v>15</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>8</v>
@@ -2467,19 +2469,19 @@
         <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>9</v>
@@ -2512,9 +2514,7 @@
       <c r="H9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
@@ -2554,22 +2554,22 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>7</v>
@@ -2578,13 +2578,13 @@
         <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
@@ -2624,46 +2624,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="S11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="U11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>32</v>
@@ -2694,49 +2694,49 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="U12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>80</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-06-30)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-29</t>
+          <t>Evolución abiertas SAT por estado — 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -679,28 +679,28 @@
         <v>8</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>5</v>
@@ -709,16 +709,16 @@
         <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="U4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -754,46 +754,46 @@
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>11</v>
@@ -825,46 +825,46 @@
         <v>23</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="P6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>22</v>
@@ -900,13 +900,13 @@
         <v>10</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>2</v>
@@ -914,28 +914,26 @@
       <c r="M7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="U7" s="6" t="inlineStr"/>
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
@@ -965,49 +963,49 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1043,35 +1041,35 @@
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
-      <c r="W9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1103,26 +1101,26 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>1</v>
@@ -1137,11 +1135,9 @@
         <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="V10" s="4" t="inlineStr"/>
       <c r="W10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1177,19 +1173,19 @@
         <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>8</v>
@@ -1198,22 +1194,22 @@
         <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>9</v>
@@ -1249,49 +1245,49 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1324,30 +1320,30 @@
         <v>1</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="O13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>4</v>
@@ -1356,13 +1352,13 @@
         <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1395,16 +1391,16 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
@@ -1419,22 +1415,22 @@
         <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>3</v>
@@ -1468,46 +1464,46 @@
         <v>11</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="L15" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>5</v>
@@ -1546,15 +1542,17 @@
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>1</v>
@@ -1609,15 +1607,17 @@
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
-      <c r="Q17" s="6" t="inlineStr"/>
-      <c r="R17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
-      <c r="U17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W17" s="6" t="n">
         <v>2</v>
@@ -1726,21 +1726,21 @@
       <c r="H20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
@@ -1749,10 +1749,10 @@
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
@@ -1761,7 +1761,7 @@
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>3</v>
@@ -1795,38 +1795,38 @@
       </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R21" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V21" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1862,43 +1862,43 @@
         <v>17</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="Q22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>11</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>15</v>
@@ -1930,46 +1930,46 @@
         <v>96</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="J23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="K23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>91</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="T23" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>82</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>79</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>82</v>
@@ -2019,7 +2019,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-29</t>
+          <t>Evolución abiertas SAT por cadena — 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -2061,77 +2061,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -2160,46 +2160,46 @@
         <v>19</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="Q4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>19</v>
@@ -2230,46 +2230,46 @@
         <v>18</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -2303,43 +2303,43 @@
         <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>5</v>
@@ -2389,7 +2389,7 @@
         <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>2</v>
@@ -2401,7 +2401,7 @@
         <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>1</v>
@@ -2438,22 +2438,22 @@
         <v>10</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>8</v>
@@ -2462,22 +2462,22 @@
         <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>12</v>
@@ -2507,9 +2507,7 @@
       <c r="G9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
@@ -2550,19 +2548,19 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>7</v>
@@ -2571,13 +2569,13 @@
         <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
@@ -2589,7 +2587,7 @@
         <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>4</v>
@@ -2620,46 +2618,46 @@
         <v>32</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>30</v>
@@ -2690,46 +2688,46 @@
         <v>96</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="I12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>92</v>
-      </c>
       <c r="J12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="S12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>82</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>79</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>82</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-01)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,13 +522,12 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-06-30</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -545,107 +544,102 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>
@@ -661,43 +655,43 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>10</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
@@ -706,21 +700,18 @@
         <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="W4" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -736,66 +727,63 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="F5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="W5" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -811,62 +799,61 @@
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="n">
+        <v>13</v>
+      </c>
       <c r="E6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="W6" s="4" t="n">
         <v>28</v>
       </c>
     </row>
@@ -882,60 +869,57 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F7" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
-      <c r="V7" s="6" t="inlineStr"/>
-      <c r="W7" s="6" t="n">
+      <c r="V7" s="6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -950,64 +934,61 @@
           <t>En cola taller</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>8</v>
-      </c>
+      <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1022,54 +1003,49 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="E9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="G9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
-      <c r="W9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1083,41 +1059,41 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
@@ -1132,14 +1108,11 @@
         <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V10" s="4" t="inlineStr"/>
-      <c r="W10" s="4" t="n">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="U10" s="4" t="inlineStr"/>
+      <c r="V10" s="4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1154,37 +1127,37 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="M11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>8</v>
@@ -1193,27 +1166,24 @@
         <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="W11" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1229,66 +1199,63 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W12" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1304,13 +1271,13 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>1</v>
@@ -1319,30 +1286,30 @@
         <v>1</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K13" s="6" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="N13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>4</v>
@@ -1351,15 +1318,12 @@
         <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="W13" s="6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1375,19 +1339,19 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H14" s="4" t="n">
         <v>5</v>
@@ -1396,10 +1360,10 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
@@ -1414,27 +1378,24 @@
         <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="W14" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1450,64 +1411,61 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q15" s="6" t="n">
+      <c r="R15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="S15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="W15" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1523,35 +1481,37 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>1</v>
@@ -1566,9 +1526,6 @@
         <v>1</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W16" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1587,13 +1544,13 @@
         <v>1</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>1</v>
@@ -1608,20 +1565,19 @@
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="inlineStr"/>
-      <c r="Q17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
-      <c r="T17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1636,16 +1592,14 @@
           <t>En reparación (online)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="E18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
@@ -1662,42 +1616,78 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
-      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Externa</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Pendiente agendar llamada</t>
+          <t>Pendiente definir servicio externo</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
-      <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
-      <c r="O19" s="6" t="inlineStr"/>
-      <c r="P19" s="6" t="inlineStr"/>
-      <c r="Q19" s="6" t="inlineStr"/>
-      <c r="R19" s="6" t="inlineStr"/>
-      <c r="S19" s="6" t="inlineStr"/>
-      <c r="T19" s="6" t="inlineStr"/>
-      <c r="U19" s="6" t="inlineStr"/>
-      <c r="V19" s="6" t="inlineStr"/>
-      <c r="W19" s="6" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V19" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1707,70 +1697,51 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Pendiente definir servicio externo</t>
+          <t>Esperando respuesta cliente a presupuesto</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="W20" s="4" t="n">
-        <v>3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1780,206 +1751,141 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Esperando respuesta cliente a presupuesto</t>
+          <t>Enviado a técnico externo</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="6" t="inlineStr"/>
+        <v>24</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>18</v>
+      </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="6" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>13</v>
+      </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" s="6" t="inlineStr"/>
-      <c r="W21" s="6" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="V21" s="6" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Externa</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Enviado a técnico externo</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr"/>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Total abiertas</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
-        <v>167</v>
-      </c>
-      <c r="D23" s="8" t="n">
+      <c r="C22" s="8" t="n">
         <v>122</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="D22" s="8" t="n">
         <v>143</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="E22" s="8" t="n">
         <v>117</v>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="F22" s="8" t="n">
         <v>129</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="G22" s="8" t="n">
         <v>96</v>
       </c>
-      <c r="I23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="J23" s="8" t="n">
+      <c r="H22" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="I22" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="K23" s="8" t="n">
+      <c r="J22" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="L23" s="8" t="n">
+      <c r="K22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="M23" s="8" t="n">
+      <c r="L22" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="N23" s="8" t="n">
+      <c r="M22" s="8" t="n">
         <v>91</v>
       </c>
-      <c r="O23" s="8" t="n">
+      <c r="N22" s="8" t="n">
         <v>91</v>
       </c>
-      <c r="P23" s="8" t="n">
+      <c r="O22" s="8" t="n">
         <v>94</v>
       </c>
-      <c r="Q23" s="8" t="n">
+      <c r="P22" s="8" t="n">
         <v>93</v>
       </c>
-      <c r="R23" s="8" t="n">
+      <c r="Q22" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="S23" s="8" t="n">
+      <c r="R22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="T23" s="8" t="n">
+      <c r="S22" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="U23" s="8" t="n">
+      <c r="T22" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="V23" s="8" t="n">
+      <c r="U22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="W23" s="8" t="n">
+      <c r="V22" s="8" t="n">
         <v>85</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1991,7 +1897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2015,13 +1921,12 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-06-30</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -2033,107 +1938,102 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>
@@ -2144,66 +2044,63 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="V4" s="4" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2214,66 +2111,63 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="V5" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2284,40 +2178,40 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
@@ -2326,7 +2220,7 @@
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>3</v>
@@ -2335,15 +2229,12 @@
         <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V6" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2353,15 +2244,15 @@
           <t>Smart Duck</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="D7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>1</v>
@@ -2388,7 +2279,7 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>2</v>
@@ -2400,7 +2291,7 @@
         <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>1</v>
@@ -2409,9 +2300,6 @@
         <v>1</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2422,37 +2310,37 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="H8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>8</v>
@@ -2461,29 +2349,26 @@
         <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="V8" s="4" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2492,10 +2377,10 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>1</v>
@@ -2504,11 +2389,9 @@
         <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
@@ -2523,7 +2406,6 @@
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
-      <c r="V9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2532,34 +2414,34 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>7</v>
@@ -2568,13 +2450,13 @@
         <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
@@ -2586,12 +2468,9 @@
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V10" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2602,66 +2481,63 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>36</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="V11" s="10" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2672,72 +2548,69 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="S12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>82</v>
-      </c>
-      <c r="V12" s="8" t="n">
         <v>85</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-02)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-01</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>5</v>
@@ -697,19 +697,19 @@
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="S4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>4</v>
@@ -745,46 +745,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -815,46 +815,46 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -887,7 +887,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
@@ -895,30 +895,30 @@
       <c r="K7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="S7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="V7" s="6" t="n">
         <v>4</v>
       </c>
@@ -952,44 +952,42 @@
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1019,34 +1017,34 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
       <c r="T9" s="6" t="inlineStr"/>
-      <c r="U9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1078,21 +1076,23 @@
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>1</v>
@@ -1107,12 +1107,12 @@
         <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="T10" s="4" t="inlineStr"/>
+      <c r="U10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
       </c>
@@ -1147,16 +1147,16 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>8</v>
@@ -1165,25 +1165,25 @@
         <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>8</v>
@@ -1219,37 +1219,37 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2</v>
@@ -1258,7 +1258,7 @@
         <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1291,24 +1291,24 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>4</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
       <c r="K13" s="6" t="inlineStr"/>
-      <c r="L13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>4</v>
@@ -1317,16 +1317,16 @@
         <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1359,10 +1359,10 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
@@ -1377,22 +1377,22 @@
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
@@ -1429,43 +1429,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>6</v>
@@ -1502,15 +1502,17 @@
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>1</v>
@@ -1524,9 +1526,7 @@
       <c r="T16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1564,18 +1564,20 @@
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
-      <c r="S17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>1</v>
@@ -1647,16 +1649,16 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>2</v>
@@ -1665,10 +1667,10 @@
         <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>2</v>
@@ -1677,7 +1679,7 @@
         <v>2</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>3</v>
@@ -1714,32 +1716,32 @@
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
     </row>
@@ -1773,43 +1775,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L21" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="M21" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>16</v>
@@ -1841,43 +1843,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>91</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="T22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="S22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="T22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="U22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>90</v>
@@ -1926,7 +1928,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-01</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -1968,72 +1970,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
     </row>
@@ -2065,40 +2067,40 @@
         <v>23</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2129,43 +2131,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>12</v>
@@ -2196,40 +2198,40 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>5</v>
@@ -2276,7 +2278,7 @@
         <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>2</v>
@@ -2288,7 +2290,7 @@
         <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>1</v>
@@ -2331,13 +2333,13 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>8</v>
@@ -2346,25 +2348,25 @@
         <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>13</v>
@@ -2435,10 +2437,10 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>7</v>
@@ -2447,13 +2449,13 @@
         <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
@@ -2465,7 +2467,7 @@
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
@@ -2502,40 +2504,40 @@
         <v>36</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="R11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>37</v>
@@ -2566,43 +2568,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="R12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-03)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-02</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -673,19 +673,19 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
@@ -694,22 +694,22 @@
         <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>12</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>24</v>
@@ -892,32 +892,32 @@
       <c r="J7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>3</v>
@@ -949,46 +949,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1022,28 +1022,28 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
-      <c r="T9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
@@ -1079,19 +1079,19 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>1</v>
@@ -1106,17 +1106,17 @@
         <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1149,13 +1149,13 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>8</v>
@@ -1164,25 +1164,25 @@
         <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>8</v>
@@ -1221,34 +1221,34 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>2</v>
@@ -1256,9 +1256,7 @@
       <c r="T12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="U12" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1290,22 +1288,22 @@
       <c r="H13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="6" t="n">
-        <v>4</v>
-      </c>
+      <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="6" t="inlineStr"/>
-      <c r="K13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="L13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>4</v>
@@ -1314,13 +1312,13 @@
         <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>3</v>
@@ -1359,7 +1357,7 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
@@ -1374,28 +1372,28 @@
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1429,43 +1427,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="S15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>10</v>
@@ -1501,15 +1499,17 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1</v>
@@ -1523,9 +1523,7 @@
       <c r="S16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
     </row>
@@ -1563,18 +1561,20 @@
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
-      <c r="R17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>1</v>
@@ -1649,43 +1649,43 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U19" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>3</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>7</v>
@@ -1715,32 +1715,32 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
@@ -1775,43 +1775,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="T21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="U21" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="U21" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>15</v>
@@ -1843,43 +1843,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>91</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="S22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="R22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="T22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>100</v>
@@ -1928,7 +1928,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-02</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -1970,72 +1970,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -2064,43 +2064,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>19</v>
@@ -2131,40 +2131,40 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>12</v>
@@ -2201,13 +2201,13 @@
         <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
@@ -2216,7 +2216,7 @@
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>3</v>
@@ -2225,10 +2225,10 @@
         <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>5</v>
@@ -2275,7 +2275,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>2</v>
@@ -2287,7 +2287,7 @@
         <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>1</v>
@@ -2330,13 +2330,13 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>8</v>
@@ -2345,28 +2345,28 @@
         <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>15</v>
@@ -2434,10 +2434,10 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>7</v>
@@ -2446,13 +2446,13 @@
         <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
@@ -2464,7 +2464,7 @@
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>4</v>
@@ -2501,43 +2501,43 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="Q11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>44</v>
@@ -2568,43 +2568,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="Q12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-04)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-03</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-04</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-03</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-05)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-04</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-05</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-04</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-06)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-05</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -673,16 +673,16 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>5</v>
@@ -691,25 +691,25 @@
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="Q4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="S4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>4</v>
@@ -745,46 +745,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="V5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -815,40 +815,40 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>24</v>
@@ -889,35 +889,35 @@
       <c r="I7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -952,43 +952,43 @@
         <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1019,28 +1019,28 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
-      <c r="S9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
@@ -1082,13 +1082,13 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>1</v>
@@ -1103,20 +1103,20 @@
         <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1149,10 +1149,10 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>8</v>
@@ -1161,25 +1161,25 @@
         <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>8</v>
@@ -1221,31 +1221,31 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>2</v>
@@ -1253,10 +1253,10 @@
       <c r="S12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V12" s="4" t="n">
         <v>1</v>
       </c>
@@ -1291,18 +1291,20 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="K13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>4</v>
@@ -1311,13 +1313,13 @@
         <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>3</v>
@@ -1371,31 +1373,31 @@
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1429,43 +1431,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="P15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="R15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>13</v>
@@ -1500,15 +1502,17 @@
       </c>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>1</v>
@@ -1522,9 +1526,7 @@
       <c r="R16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
@@ -1562,18 +1564,20 @@
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
-      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>1</v>
@@ -1651,40 +1655,40 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T19" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>3</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>7</v>
@@ -1716,35 +1720,37 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1779,43 +1785,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="S21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="T21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="T21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="U21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>14</v>
@@ -1847,46 +1853,46 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="K22" s="8" t="n">
         <v>91</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="R22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="Q22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="R22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="S22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1932,7 +1938,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-05</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -1974,72 +1980,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -2068,40 +2074,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>19</v>
@@ -2135,46 +2141,46 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -2202,34 +2208,34 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>5</v>
@@ -2238,7 +2244,7 @@
         <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>6</v>
@@ -2276,7 +2282,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>2</v>
@@ -2288,7 +2294,7 @@
         <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>1</v>
@@ -2337,7 +2343,7 @@
         <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>8</v>
@@ -2346,31 +2352,31 @@
         <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>16</v>
@@ -2438,7 +2444,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>7</v>
@@ -2447,13 +2453,13 @@
         <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
@@ -2465,7 +2471,7 @@
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
@@ -2505,43 +2511,43 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>33</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>27</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="P11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>45</v>
@@ -2572,46 +2578,46 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="P12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="R12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-07)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-06</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -676,10 +676,10 @@
         <v>2</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
@@ -688,25 +688,25 @@
         <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>4</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>13</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>22</v>
@@ -886,38 +886,38 @@
       <c r="H7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>7</v>
@@ -949,43 +949,43 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -1018,33 +1018,31 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1077,13 +1075,13 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>1</v>
@@ -1098,20 +1096,20 @@
         <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="Q10" s="4" t="inlineStr"/>
+      <c r="R10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1147,7 +1145,7 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>8</v>
@@ -1156,25 +1154,25 @@
         <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>8</v>
@@ -1183,7 +1181,7 @@
         <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>11</v>
@@ -1219,28 +1217,28 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>2</v>
@@ -1248,15 +1246,15 @@
       <c r="R12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="S12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1288,18 +1286,20 @@
       <c r="H13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="J13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>4</v>
@@ -1308,13 +1308,13 @@
         <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>3</v>
@@ -1326,7 +1326,7 @@
         <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1368,34 +1368,34 @@
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>3</v>
@@ -1429,43 +1429,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="O15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>4</v>
@@ -1499,15 +1499,17 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>1</v>
@@ -1521,9 +1523,7 @@
       <c r="Q16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
@@ -1561,18 +1561,20 @@
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>1</v>
@@ -1653,7 +1655,7 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>2</v>
@@ -1662,10 +1664,10 @@
         <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>2</v>
@@ -1674,7 +1676,7 @@
         <v>2</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>3</v>
@@ -1683,13 +1685,13 @@
         <v>3</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>10</v>
@@ -1722,32 +1724,32 @@
         <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1783,43 +1785,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="S21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="T21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>13</v>
@@ -1851,43 +1853,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>91</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="P22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="R22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>102</v>
@@ -1936,7 +1938,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-06</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -1978,72 +1980,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -2072,43 +2074,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>21</v>
@@ -2142,40 +2144,40 @@
         <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
@@ -2206,43 +2208,43 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>5</v>
@@ -2277,7 +2279,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>2</v>
@@ -2289,7 +2291,7 @@
         <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>1</v>
@@ -2338,7 +2340,7 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>8</v>
@@ -2347,34 +2349,34 @@
         <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>16</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>13</v>
@@ -2414,7 +2416,9 @@
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
       <c r="S9" s="6" t="inlineStr"/>
-      <c r="T9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U9" s="6" t="n">
         <v>1</v>
       </c>
@@ -2450,13 +2454,13 @@
         <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
@@ -2468,7 +2472,7 @@
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>4</v>
@@ -2480,7 +2484,7 @@
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>3</v>
@@ -2511,43 +2515,43 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>44</v>
@@ -2578,43 +2582,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>91</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>102</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-08)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-07</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
     </row>
@@ -673,10 +673,10 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
@@ -685,31 +685,31 @@
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>3</v>
@@ -748,40 +748,40 @@
         <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="O5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="T6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>24</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>22</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>24</v>
@@ -886,38 +886,40 @@
       <c r="H7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>4</v>
@@ -949,46 +951,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="U8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="V8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1018,33 +1020,35 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr"/>
+      <c r="U9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1077,10 +1081,10 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>1</v>
@@ -1095,24 +1099,22 @@
         <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="P10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U10" s="4" t="inlineStr"/>
       <c r="V10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1151,25 +1153,25 @@
         <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>8</v>
@@ -1178,7 +1180,7 @@
         <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>11</v>
@@ -1217,25 +1219,25 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
@@ -1243,15 +1245,15 @@
       <c r="Q12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="R12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>3</v>
@@ -1290,13 +1292,13 @@
         <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>4</v>
@@ -1305,13 +1307,13 @@
         <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>3</v>
@@ -1323,7 +1325,7 @@
         <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>2</v>
@@ -1365,37 +1367,37 @@
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1429,43 +1431,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="N15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="S15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>8</v>
@@ -1498,15 +1500,17 @@
       <c r="H16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>1</v>
@@ -1520,9 +1524,7 @@
       <c r="P16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
@@ -1560,18 +1562,20 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>1</v>
@@ -1661,10 +1665,10 @@
         <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>2</v>
@@ -1673,7 +1677,7 @@
         <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>3</v>
@@ -1682,16 +1686,16 @@
         <v>3</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="U19" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>7</v>
@@ -1721,32 +1725,32 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
@@ -1785,43 +1789,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="R21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="S21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>18</v>
@@ -1856,40 +1860,40 @@
         <v>91</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="P22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="O22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="Q22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>107</v>
@@ -1938,7 +1942,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-07</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -1980,72 +1984,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
     </row>
@@ -2074,43 +2078,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>23</v>
@@ -2141,40 +2145,40 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>14</v>
@@ -2208,7 +2212,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
@@ -2217,7 +2221,7 @@
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>3</v>
@@ -2226,10 +2230,10 @@
         <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>5</v>
@@ -2238,10 +2242,10 @@
         <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>5</v>
@@ -2276,7 +2280,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
@@ -2288,7 +2292,7 @@
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>1</v>
@@ -2346,37 +2350,37 @@
         <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>12</v>
@@ -2415,9 +2419,11 @@
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
       <c r="R9" s="6" t="inlineStr"/>
-      <c r="S9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>4</v>
@@ -2451,13 +2457,13 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
@@ -2469,7 +2475,7 @@
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>4</v>
@@ -2481,7 +2487,7 @@
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>3</v>
@@ -2515,43 +2521,43 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="N11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="S11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>45</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>45</v>
@@ -2585,40 +2591,40 @@
         <v>91</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>107</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-09)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-08</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
@@ -682,34 +682,34 @@
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>4</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>13</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="S6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>27</v>
@@ -887,39 +887,39 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>3</v>
@@ -951,43 +951,43 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
@@ -1021,34 +1021,34 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1081,7 +1081,7 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
@@ -1096,27 +1096,27 @@
         <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="T10" s="4" t="inlineStr"/>
+      <c r="U10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1152,25 +1152,25 @@
         <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>8</v>
@@ -1179,13 +1179,13 @@
         <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>13</v>
@@ -1224,19 +1224,19 @@
         <v>6</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
@@ -1244,18 +1244,18 @@
       <c r="P12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="Q12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>4</v>
@@ -1291,13 +1291,13 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>4</v>
@@ -1306,13 +1306,13 @@
         <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>3</v>
@@ -1324,7 +1324,7 @@
         <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>2</v>
@@ -1366,40 +1366,40 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>1</v>
@@ -1433,43 +1433,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="M15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>7</v>
@@ -1503,13 +1503,13 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L16" s="4" t="n">
         <v>1</v>
@@ -1523,9 +1523,7 @@
       <c r="O16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
@@ -1563,18 +1561,20 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
@@ -1664,10 +1664,10 @@
         <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>2</v>
@@ -1676,7 +1676,7 @@
         <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>3</v>
@@ -1685,19 +1685,19 @@
         <v>3</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="T19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="U19" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>8</v>
@@ -1727,35 +1727,35 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>3</v>
@@ -1791,40 +1791,40 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="Q21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="R21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>18</v>
@@ -1859,43 +1859,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="O22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="N22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="P22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>109</v>
@@ -1944,7 +1944,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-08</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -1986,72 +1986,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>
@@ -2080,40 +2080,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>26</v>
-      </c>
       <c r="J4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>23</v>
@@ -2147,43 +2147,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>15</v>
@@ -2220,7 +2220,7 @@
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>3</v>
@@ -2229,10 +2229,10 @@
         <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>5</v>
@@ -2241,10 +2241,10 @@
         <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>5</v>
@@ -2279,7 +2279,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>2</v>
@@ -2291,7 +2291,7 @@
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>1</v>
@@ -2314,9 +2314,7 @@
       <c r="S7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2347,40 +2345,40 @@
         <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="P8" s="4" t="n">
+      <c r="T8" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>13</v>
@@ -2418,9 +2416,11 @@
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>4</v>
@@ -2454,13 +2454,13 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
@@ -2472,7 +2472,7 @@
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>4</v>
@@ -2484,13 +2484,13 @@
         <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2521,40 +2521,40 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>33</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="R11" s="10" t="n">
+      <c r="S11" s="10" t="n">
         <v>45</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>45</v>
@@ -2588,43 +2588,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="O12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>109</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-10)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-09</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -679,37 +679,37 @@
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>3</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="M5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
+      <c r="T5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="R6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>22</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>27</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>22</v>
@@ -890,39 +890,39 @@
         <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -951,43 +951,43 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="S8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>6</v>
@@ -1021,28 +1021,28 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="inlineStr"/>
+      <c r="S9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -1093,30 +1093,30 @@
         <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1149,25 +1149,25 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>8</v>
@@ -1176,16 +1176,16 @@
         <v>8</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>12</v>
@@ -1221,19 +1221,19 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
@@ -1241,21 +1241,21 @@
       <c r="O12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="P12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
@@ -1291,10 +1291,10 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>4</v>
@@ -1303,13 +1303,13 @@
         <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>3</v>
@@ -1321,13 +1321,13 @@
         <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
@@ -1363,40 +1363,40 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>1</v>
@@ -1433,43 +1433,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="L15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="T15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>8</v>
@@ -1506,7 +1506,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>1</v>
@@ -1520,9 +1520,7 @@
       <c r="N16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
@@ -1560,18 +1558,20 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>1</v>
@@ -1628,7 +1628,9 @@
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
+      <c r="U18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1663,10 +1665,10 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>2</v>
@@ -1675,7 +1677,7 @@
         <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>3</v>
@@ -1684,25 +1686,25 @@
         <v>3</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="S19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="T19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="U19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="V19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -1728,39 +1730,39 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
-      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1793,43 +1795,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="O21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="P21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="Q21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>20</v>
@@ -1861,40 +1863,40 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="N22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="M22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="O22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U22" s="8" t="n">
         <v>109</v>
@@ -1946,7 +1948,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-09</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -1988,72 +1990,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -2082,43 +2084,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>24</v>
@@ -2149,43 +2151,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
@@ -2219,7 +2221,7 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -2228,10 +2230,10 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>5</v>
@@ -2240,10 +2242,10 @@
         <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>5</v>
@@ -2290,7 +2292,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>1</v>
@@ -2313,9 +2315,7 @@
       <c r="R7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
     </row>
@@ -2344,43 +2344,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="S8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>11</v>
@@ -2417,9 +2417,11 @@
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="6" t="inlineStr"/>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>4</v>
@@ -2459,7 +2461,7 @@
         <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
@@ -2471,7 +2473,7 @@
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>4</v>
@@ -2483,13 +2485,13 @@
         <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
@@ -2526,34 +2528,34 @@
         <v>33</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="Q11" s="10" t="n">
+      <c r="R11" s="10" t="n">
         <v>45</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>45</v>
@@ -2590,40 +2592,40 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="N12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>109</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-11)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-10</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-11</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-10</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-12)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-11</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-12</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-11</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-13)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-12</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -676,37 +676,37 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>3</v>
@@ -745,40 +745,40 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="L5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
+      <c r="S5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>11</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="S6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>21</v>
@@ -887,39 +887,39 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>3</v>
@@ -954,43 +954,43 @@
         <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1020,35 +1020,35 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1090,30 +1090,30 @@
         <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>3</v>
@@ -1152,19 +1152,19 @@
         <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>8</v>
@@ -1173,19 +1173,19 @@
         <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>12</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>11</v>
@@ -1221,16 +1221,16 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
@@ -1238,21 +1238,21 @@
       <c r="N12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="O12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>2</v>
@@ -1291,7 +1291,7 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>4</v>
@@ -1300,13 +1300,13 @@
         <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>3</v>
@@ -1318,19 +1318,19 @@
         <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1363,37 +1363,37 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>1</v>
@@ -1402,7 +1402,7 @@
         <v>1</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1433,43 +1433,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="K15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="P15" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="T15" s="6" t="n">
+      <c r="U15" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>8</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>7</v>
@@ -1503,7 +1503,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>1</v>
@@ -1517,9 +1517,7 @@
       <c r="M16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -1558,17 +1556,17 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O17" s="6" t="n">
         <v>1</v>
@@ -1627,7 +1625,9 @@
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>2</v>
@@ -1674,7 +1674,7 @@
         <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>3</v>
@@ -1683,25 +1683,25 @@
         <v>3</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="Q19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="R19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="S19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="T19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="U19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>6</v>
@@ -1730,36 +1730,38 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1795,43 +1797,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="O21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="P21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>22</v>
@@ -1863,43 +1865,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="M22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="L22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="N22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>107</v>
@@ -1948,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-12</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -1990,72 +1992,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -2084,43 +2086,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>22</v>
@@ -2151,40 +2153,40 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>16</v>
@@ -2218,7 +2220,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>3</v>
@@ -2227,10 +2229,10 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>5</v>
@@ -2239,10 +2241,10 @@
         <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>5</v>
@@ -2289,7 +2291,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>1</v>
@@ -2312,9 +2314,7 @@
       <c r="Q7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
@@ -2344,43 +2344,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="R8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="R8" s="4" t="n">
+      <c r="S8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>12</v>
@@ -2416,9 +2416,11 @@
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>4</v>
@@ -2458,7 +2460,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
@@ -2470,7 +2472,7 @@
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>4</v>
@@ -2482,13 +2484,13 @@
         <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>4</v>
@@ -2525,34 +2527,34 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>29</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="P11" s="10" t="n">
+      <c r="Q11" s="10" t="n">
         <v>45</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>45</v>
@@ -2561,7 +2563,7 @@
         <v>45</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>44</v>
@@ -2592,43 +2594,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="M12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="S12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>107</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-14)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-13</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="K4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="M4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>6</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
+      <c r="R5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>9</v>
@@ -818,40 +818,40 @@
         <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="R6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>18</v>
@@ -887,39 +887,39 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>9</v>
@@ -951,43 +951,43 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" s="4" t="n">
+      <c r="R8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="R8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>4</v>
@@ -1024,28 +1024,30 @@
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>4</v>
@@ -1087,33 +1089,33 @@
         <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="Q10" s="4" t="inlineStr"/>
+      <c r="R10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -1149,19 +1151,19 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>8</v>
@@ -1170,22 +1172,22 @@
         <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="S11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="U11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>10</v>
@@ -1221,13 +1223,13 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
@@ -1235,21 +1237,21 @@
       <c r="M12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="N12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2</v>
@@ -1297,13 +1299,13 @@
         <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3</v>
@@ -1315,19 +1317,19 @@
         <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>1</v>
@@ -1363,34 +1365,34 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>1</v>
@@ -1399,7 +1401,7 @@
         <v>1</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1433,43 +1435,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="O15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>10</v>
@@ -1514,9 +1516,7 @@
       <c r="L16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
@@ -1558,12 +1558,14 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1</v>
@@ -1624,7 +1626,9 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1671,7 +1675,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>3</v>
@@ -1680,25 +1684,25 @@
         <v>3</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="Q19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="R19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="S19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="T19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>6</v>
@@ -1734,34 +1738,34 @@
         <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>4</v>
@@ -1797,43 +1801,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="M21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="O21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>16</v>
@@ -1865,43 +1869,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="L22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="K22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="M22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="S22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>108</v>
@@ -1950,7 +1954,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-13</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1996,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -2089,37 +2093,37 @@
         <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>22</v>
@@ -2153,43 +2157,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>15</v>
@@ -2226,10 +2230,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>5</v>
@@ -2238,13 +2242,13 @@
         <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="P6" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>6</v>
@@ -2288,7 +2292,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
@@ -2311,9 +2315,7 @@
       <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
@@ -2347,40 +2349,40 @@
         <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="Q8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="P8" s="4" t="n">
+      <c r="R8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>13</v>
@@ -2415,9 +2417,11 @@
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>4</v>
@@ -2429,7 +2433,7 @@
         <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -2469,7 +2473,7 @@
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>4</v>
@@ -2481,13 +2485,13 @@
         <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
@@ -2496,7 +2500,7 @@
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>3</v>
@@ -2527,28 +2531,28 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>44</v>
@@ -2560,10 +2564,10 @@
         <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>47</v>
@@ -2594,43 +2598,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="K12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="L12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>108</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-15)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-14</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="L4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>7</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
+      <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>10</v>
@@ -815,40 +815,40 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>18</v>
@@ -887,39 +887,39 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>12</v>
@@ -951,46 +951,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P8" s="4" t="n">
+      <c r="Q8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1023,34 +1023,36 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1086,36 +1088,36 @@
         <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="P10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>7</v>
@@ -1154,13 +1156,13 @@
         <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>8</v>
@@ -1169,25 +1171,25 @@
         <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="T11" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>9</v>
@@ -1223,10 +1225,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
@@ -1234,21 +1236,21 @@
       <c r="L12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>2</v>
@@ -1257,10 +1259,10 @@
         <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1296,13 +1298,13 @@
         <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>3</v>
@@ -1314,25 +1316,25 @@
         <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1365,31 +1367,31 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>1</v>
@@ -1398,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>2</v>
@@ -1435,43 +1437,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>10</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="N15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>9</v>
@@ -1513,9 +1515,7 @@
       <c r="K16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
@@ -1557,12 +1557,14 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
@@ -1625,16 +1627,16 @@
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1670,7 +1672,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>3</v>
@@ -1679,31 +1681,31 @@
         <v>3</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="P19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="Q19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="R19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="S19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>4</v>
@@ -1733,34 +1735,34 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>4</v>
@@ -1799,43 +1801,43 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="N21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>12</v>
@@ -1867,43 +1869,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="K22" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="J22" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="L22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>105</v>
@@ -1952,7 +1954,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-14</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -1994,72 +1996,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
@@ -2088,43 +2090,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2155,43 +2157,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
@@ -2225,10 +2227,10 @@
         <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>5</v>
@@ -2237,13 +2239,13 @@
         <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>6</v>
@@ -2287,7 +2289,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>1</v>
@@ -2310,9 +2312,7 @@
       <c r="O7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
@@ -2344,43 +2344,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>9</v>
@@ -2414,9 +2414,11 @@
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>4</v>
@@ -2428,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
@@ -2468,7 +2470,7 @@
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
@@ -2480,13 +2482,13 @@
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>4</v>
@@ -2495,10 +2497,10 @@
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2529,25 +2531,25 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>44</v>
@@ -2559,13 +2561,13 @@
         <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>50</v>
@@ -2596,43 +2598,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>79</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>105</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-16)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-15</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-16</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="K4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>6</v>
@@ -745,40 +745,40 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
+      <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>10</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="P6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="R6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>19</v>
@@ -886,40 +886,40 @@
       <c r="H7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>6</v>
@@ -951,46 +951,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1022,37 +1022,39 @@
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1085,42 +1087,42 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1153,13 +1155,13 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>8</v>
@@ -1168,28 +1170,28 @@
         <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="Q11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R11" s="6" t="n">
+      <c r="S11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>12</v>
@@ -1225,7 +1227,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
@@ -1233,21 +1235,21 @@
       <c r="K12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="L12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>2</v>
@@ -1256,13 +1258,13 @@
         <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V12" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1295,13 +1297,13 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>3</v>
@@ -1313,28 +1315,28 @@
         <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1370,25 +1372,25 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>1</v>
@@ -1397,7 +1399,7 @@
         <v>1</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>2</v>
@@ -1440,40 +1442,40 @@
         <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="M15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="T15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>10</v>
@@ -1512,9 +1514,7 @@
       <c r="J16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1524,7 +1524,9 @@
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="V16" s="4" t="n">
         <v>2</v>
       </c>
@@ -1558,12 +1560,14 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>1</v>
@@ -1628,16 +1632,16 @@
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
@@ -1671,7 +1675,7 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>3</v>
@@ -1680,34 +1684,34 @@
         <v>3</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="O19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="P19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="Q19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="R19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>3</v>
@@ -1737,37 +1741,37 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>5</v>
@@ -1806,37 +1810,37 @@
         <v>11</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="M21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>12</v>
@@ -1871,43 +1875,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="Q22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>106</v>
@@ -1956,7 +1960,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-15</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-16</t>
         </is>
       </c>
     </row>
@@ -1998,72 +2002,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
@@ -2095,40 +2099,40 @@
         <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>19</v>
@@ -2159,40 +2163,40 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>16</v>
@@ -2226,10 +2230,10 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>5</v>
@@ -2238,13 +2242,13 @@
         <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="N6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>6</v>
@@ -2262,7 +2266,7 @@
         <v>6</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>8</v>
@@ -2311,9 +2315,7 @@
       <c r="N7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
@@ -2346,40 +2348,40 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>9</v>
@@ -2415,9 +2417,11 @@
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>4</v>
@@ -2429,7 +2433,7 @@
         <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
@@ -2469,7 +2473,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
@@ -2481,13 +2485,13 @@
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>4</v>
@@ -2496,10 +2500,10 @@
         <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
@@ -2533,22 +2537,22 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>44</v>
@@ -2560,16 +2564,16 @@
         <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>48</v>
@@ -2600,43 +2604,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>106</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-17)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-16</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-17</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
@@ -673,40 +673,40 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>6</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>17</v>
@@ -887,36 +887,38 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>6</v>
@@ -954,40 +956,40 @@
         <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
@@ -1021,37 +1023,39 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -1086,40 +1090,40 @@
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1155,10 +1159,10 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>8</v>
@@ -1167,31 +1171,31 @@
         <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="P11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q11" s="6" t="n">
+      <c r="R11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="T11" s="6" t="n">
+      <c r="U11" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>12</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>9</v>
@@ -1232,21 +1236,21 @@
       <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>2</v>
@@ -1255,13 +1259,13 @@
         <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U12" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>5</v>
@@ -1300,7 +1304,7 @@
         <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>3</v>
@@ -1312,28 +1316,28 @@
         <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
@@ -1369,25 +1373,25 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>1</v>
@@ -1396,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>2</v>
@@ -1439,43 +1443,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="S15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="T15" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>12</v>
@@ -1511,9 +1515,7 @@
       <c r="I16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
@@ -1523,7 +1525,9 @@
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
-      <c r="T16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="U16" s="4" t="n">
         <v>2</v>
       </c>
@@ -1561,10 +1565,10 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>1</v>
@@ -1631,16 +1635,16 @@
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1681,37 +1685,37 @@
         <v>3</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="N19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="O19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="P19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="Q19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>4</v>
@@ -1740,38 +1744,38 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>3</v>
@@ -1807,37 +1811,37 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="L21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>12</v>
@@ -1875,43 +1879,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>104</v>
@@ -1960,7 +1964,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-16</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-17</t>
         </is>
       </c>
     </row>
@@ -2002,72 +2006,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
@@ -2096,43 +2100,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2163,43 +2167,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>15</v>
@@ -2230,7 +2234,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>5</v>
@@ -2239,13 +2243,13 @@
         <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>6</v>
@@ -2263,10 +2267,10 @@
         <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>7</v>
@@ -2312,9 +2316,7 @@
       <c r="M7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
@@ -2348,43 +2350,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>11</v>
@@ -2416,9 +2418,11 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>4</v>
@@ -2430,7 +2434,7 @@
         <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
@@ -2470,43 +2474,43 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2537,19 +2541,19 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>44</v>
@@ -2561,19 +2565,19 @@
         <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>46</v>
@@ -2604,43 +2608,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>104</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-18)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-17</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-18</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-17</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-19)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-18</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-19</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-18</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-20)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-19</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-20</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -673,43 +673,43 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="K4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>5</v>
@@ -745,43 +745,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>8</v>
@@ -815,43 +815,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="P6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>16</v>
@@ -886,42 +886,44 @@
       <c r="H7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>8</v>
@@ -953,43 +955,43 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>8</v>
@@ -1022,40 +1024,42 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
@@ -1090,37 +1094,39 @@
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>2</v>
@@ -1159,7 +1165,7 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>8</v>
@@ -1168,34 +1174,34 @@
         <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="S11" s="6" t="n">
+      <c r="T11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="T11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="U11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
@@ -1233,21 +1239,21 @@
       <c r="I12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
@@ -1256,19 +1262,19 @@
         <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="T12" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1301,7 +1307,7 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>3</v>
@@ -1313,34 +1319,34 @@
         <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1376,19 +1382,19 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>1</v>
@@ -1397,7 +1403,7 @@
         <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>2</v>
@@ -1409,7 +1415,7 @@
         <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>3</v>
@@ -1443,43 +1449,43 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="R15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>11</v>
@@ -1512,9 +1518,7 @@
       <c r="H16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
@@ -1524,12 +1528,14 @@
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V16" s="4" t="n">
         <v>1</v>
@@ -1565,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
@@ -1634,16 +1640,16 @@
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
@@ -1682,43 +1688,43 @@
         <v>3</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="M19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="N19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="O19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="P19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1746,36 +1752,38 @@
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1811,34 +1819,34 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J21" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="K21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>12</v>
@@ -1847,10 +1855,10 @@
         <v>12</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
@@ -1879,43 +1887,43 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>100</v>
@@ -1964,7 +1972,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-19</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-20</t>
         </is>
       </c>
     </row>
@@ -2006,72 +2014,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -2100,40 +2108,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>18</v>
@@ -2167,46 +2175,46 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2240,37 +2248,37 @@
         <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="L6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>5</v>
@@ -2313,9 +2321,7 @@
       <c r="L7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
@@ -2323,7 +2329,9 @@
       <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2350,43 +2358,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="L8" s="4" t="n">
+      <c r="N8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>10</v>
@@ -2417,9 +2425,11 @@
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>4</v>
@@ -2431,7 +2441,7 @@
         <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
@@ -2483,13 +2493,13 @@
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>4</v>
@@ -2498,19 +2508,19 @@
         <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2541,16 +2551,16 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>44</v>
@@ -2562,22 +2572,22 @@
         <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>46</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>47</v>
@@ -2608,43 +2618,43 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-21)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:W22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,13 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-20</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-21</t>
         </is>
       </c>
     </row>
@@ -642,6 +643,11 @@
           <t>2026-07-20</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -714,6 +720,9 @@
       <c r="V4" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="W4" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -784,6 +793,9 @@
         <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="W5" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -856,6 +868,9 @@
       <c r="V6" s="4" t="n">
         <v>14</v>
       </c>
+      <c r="W6" s="4" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -926,6 +941,9 @@
         <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="W7" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -996,6 +1014,9 @@
       <c r="V8" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="W8" s="4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1064,6 +1085,9 @@
       <c r="V9" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="W9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1134,6 +1158,9 @@
       <c r="V10" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W10" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1206,6 +1233,9 @@
       <c r="V11" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="W11" s="6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1276,6 +1306,9 @@
       <c r="V12" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="W12" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1348,6 +1381,9 @@
       <c r="V13" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="W13" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1418,6 +1454,9 @@
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="W14" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1488,6 +1527,9 @@
         <v>11</v>
       </c>
       <c r="V15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1540,6 +1582,9 @@
       <c r="V16" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="W16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1610,6 +1655,9 @@
         <v>1</v>
       </c>
       <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1654,6 +1702,7 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1724,6 +1773,9 @@
         <v>4</v>
       </c>
       <c r="V19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="W19" s="6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1788,6 +1840,9 @@
       <c r="V20" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="W20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1858,6 +1913,9 @@
         <v>14</v>
       </c>
       <c r="V21" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="W21" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1928,10 +1986,13 @@
       <c r="V22" s="8" t="n">
         <v>91</v>
       </c>
+      <c r="W22" s="8" t="n">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1943,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1967,12 +2028,13 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-20</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-21</t>
         </is>
       </c>
     </row>
@@ -2082,6 +2144,11 @@
           <t>2026-07-20</t>
         </is>
       </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2149,6 +2216,9 @@
       <c r="U4" s="4" t="n">
         <v>14</v>
       </c>
+      <c r="V4" s="4" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2216,6 +2286,9 @@
       <c r="U5" s="6" t="n">
         <v>14</v>
       </c>
+      <c r="V5" s="6" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2281,6 +2354,9 @@
         <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2330,6 +2406,7 @@
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" s="6" t="inlineStr"/>
+      <c r="V7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2395,6 +2472,9 @@
         <v>10</v>
       </c>
       <c r="U8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2456,6 +2536,9 @@
       <c r="U9" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="V9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2523,6 +2606,9 @@
       <c r="U10" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="V10" s="4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2590,6 +2676,9 @@
       <c r="U11" s="10" t="n">
         <v>44</v>
       </c>
+      <c r="V11" s="10" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2657,10 +2746,13 @@
       <c r="U12" s="8" t="n">
         <v>91</v>
       </c>
+      <c r="V12" s="8" t="n">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-22)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-21</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-22</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -754,46 +754,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>16</v>
@@ -827,43 +827,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>14</v>
@@ -902,46 +902,46 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>5</v>
@@ -973,46 +973,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="M8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>9</v>
@@ -1046,44 +1046,44 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>4</v>
@@ -1119,44 +1119,44 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1198,34 +1198,34 @@
         <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O11" s="6" t="n">
+      <c r="P11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="P11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="R11" s="6" t="n">
+      <c r="S11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="S11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
@@ -1266,21 +1266,21 @@
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
@@ -1289,25 +1289,25 @@
         <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1349,39 +1349,39 @@
         <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V13" s="6" t="inlineStr"/>
+      <c r="W13" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1413,19 +1413,19 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
@@ -1434,7 +1434,7 @@
         <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>2</v>
@@ -1446,13 +1446,13 @@
         <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>3</v>
@@ -1486,46 +1486,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="Q15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="R15" s="6" t="n">
+      <c r="S15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="T15" s="6" t="n">
+      <c r="V15" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>12</v>
@@ -1567,12 +1567,14 @@
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
-      <c r="R16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="S16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U16" s="4" t="n">
         <v>1</v>
@@ -1685,16 +1687,16 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
@@ -1732,43 +1734,43 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="L19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="M19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="N19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="O19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>2</v>
@@ -1801,39 +1803,41 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
@@ -1872,31 +1876,31 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>12</v>
@@ -1905,13 +1909,13 @@
         <v>12</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>7</v>
@@ -1943,46 +1947,46 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="N22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>92</v>
@@ -2032,7 +2036,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-21</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-22</t>
         </is>
       </c>
     </row>
@@ -2074,77 +2078,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -2173,46 +2177,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>15</v>
@@ -2246,43 +2250,43 @@
         <v>12</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2316,13 +2320,13 @@
         <v>5</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>6</v>
@@ -2340,16 +2344,16 @@
         <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2392,9 +2396,7 @@
       <c r="K7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
@@ -2431,46 +2433,46 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="K8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="O8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>4</v>
@@ -2500,9 +2502,11 @@
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>4</v>
@@ -2514,7 +2518,7 @@
         <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
@@ -2569,13 +2573,13 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>4</v>
@@ -2584,22 +2588,22 @@
         <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2633,13 +2637,13 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>44</v>
@@ -2651,28 +2655,28 @@
         <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="P11" s="10" t="n">
+      <c r="U11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>47</v>
@@ -2703,46 +2707,46 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>92</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-23)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-22</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-23</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="U4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="V4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -754,46 +754,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>12</v>
@@ -830,43 +830,43 @@
         <v>24</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="N6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>18</v>
@@ -902,46 +902,46 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>9</v>
@@ -976,46 +976,46 @@
         <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1048,45 +1048,45 @@
       <c r="I9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1122,38 +1122,38 @@
         <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1195,34 +1195,34 @@
         <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="N11" s="6" t="n">
+      <c r="O11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q11" s="6" t="n">
+      <c r="R11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
@@ -1266,18 +1266,20 @@
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
@@ -1286,29 +1288,27 @@
         <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="R12" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="W12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1346,41 +1346,41 @@
         <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="P13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U13" s="6" t="inlineStr"/>
+      <c r="V13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1413,16 +1413,16 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
@@ -1431,7 +1431,7 @@
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>2</v>
@@ -1443,16 +1443,16 @@
         <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>4</v>
@@ -1486,46 +1486,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="P15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q15" s="6" t="n">
+      <c r="R15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="S15" s="6" t="n">
+      <c r="U15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="T15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>14</v>
@@ -1566,12 +1566,14 @@
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="R16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>1</v>
@@ -1654,9 +1656,7 @@
       <c r="U17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1684,16 +1684,16 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
@@ -1735,37 +1735,37 @@
         <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="L19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="M19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="N19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>2</v>
@@ -1774,7 +1774,7 @@
         <v>2</v>
       </c>
       <c r="W19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1800,39 +1800,41 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
@@ -1874,28 +1876,28 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>12</v>
@@ -1904,19 +1906,19 @@
         <v>12</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="V21" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="W21" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="W21" s="6" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="22">
@@ -1945,49 +1947,49 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="V22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="W22" s="8" t="n">
         <v>92</v>
-      </c>
-      <c r="W22" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2034,7 +2036,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-22</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2076,77 +2078,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2178,43 +2180,43 @@
         <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>14</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>14</v>
@@ -2245,46 +2247,46 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>16</v>
@@ -2315,13 +2317,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>6</v>
@@ -2339,22 +2341,22 @@
         <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>3</v>
@@ -2391,9 +2393,7 @@
       <c r="J7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
@@ -2431,49 +2431,49 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="R8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="V8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2499,9 +2499,11 @@
       </c>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>4</v>
@@ -2513,7 +2515,7 @@
         <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
@@ -2568,13 +2570,13 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>4</v>
@@ -2583,22 +2585,22 @@
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
@@ -2635,10 +2637,10 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>44</v>
@@ -2650,28 +2652,28 @@
         <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="O11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>47</v>
@@ -2705,49 +2707,49 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>92</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-24)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-23</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-24</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>10</v>
@@ -754,43 +754,43 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>12</v>
@@ -827,46 +827,46 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="M6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>17</v>
@@ -902,46 +902,46 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>10</v>
@@ -973,49 +973,49 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="K8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1045,48 +1045,48 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1119,47 +1119,47 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1192,34 +1192,34 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="M11" s="6" t="n">
+      <c r="N11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="Q11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="R11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
@@ -1231,7 +1231,7 @@
         <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>8</v>
@@ -1267,16 +1267,16 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
@@ -1285,29 +1285,27 @@
         <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V12" s="4" t="inlineStr"/>
       <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1343,42 +1341,40 @@
         <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U13" s="6" t="inlineStr"/>
-      <c r="V13" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T13" s="6" t="inlineStr"/>
+      <c r="U13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1411,13 +1407,13 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
@@ -1426,7 +1422,7 @@
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>2</v>
@@ -1438,19 +1434,19 @@
         <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>3</v>
@@ -1484,46 +1480,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="M15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="Q15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="R15" s="6" t="n">
+      <c r="T15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>17</v>
@@ -1563,12 +1559,14 @@
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="Q16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>1</v>
@@ -1651,9 +1649,7 @@
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
@@ -1681,16 +1677,16 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
@@ -1730,37 +1726,37 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="J19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J19" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="K19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="L19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="M19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>2</v>
@@ -1769,7 +1765,7 @@
         <v>2</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W19" s="6" t="n">
         <v>1</v>
@@ -1799,37 +1795,37 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>1</v>
@@ -1838,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>2</v>
@@ -1874,25 +1870,25 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>12</v>
@@ -1901,16 +1897,16 @@
         <v>12</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>8</v>
@@ -1945,46 +1941,46 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>99</v>
@@ -2034,7 +2030,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-23</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2076,77 +2072,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2175,46 +2171,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>19</v>
@@ -2245,43 +2241,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
@@ -2315,10 +2311,10 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>6</v>
@@ -2336,22 +2332,22 @@
         <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2388,9 +2384,7 @@
       <c r="I7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
@@ -2401,7 +2395,9 @@
       <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
       <c r="T7" s="6" t="inlineStr"/>
-      <c r="U7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2431,46 +2427,46 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="N8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -2498,9 +2494,11 @@
         <v>5</v>
       </c>
       <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>4</v>
@@ -2512,7 +2510,7 @@
         <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
@@ -2567,13 +2565,13 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
@@ -2582,22 +2580,22 @@
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
@@ -2637,7 +2635,7 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>44</v>
@@ -2649,34 +2647,34 @@
         <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="N11" s="10" t="n">
+      <c r="S11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>47</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>48</v>
@@ -2707,46 +2705,46 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>99</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-25)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-24</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-25</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-24</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-26)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-25</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-26</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-25</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-27)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-26</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-27</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>6</v>
@@ -754,46 +754,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>10</v>
@@ -827,46 +827,46 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>27</v>
-      </c>
       <c r="L6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>23</v>
@@ -902,46 +902,46 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>3</v>
@@ -973,46 +973,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>8</v>
@@ -1045,45 +1045,47 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>2</v>
@@ -1118,45 +1120,45 @@
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>1</v>
@@ -1195,28 +1197,28 @@
         <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="L11" s="6" t="n">
+      <c r="M11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O11" s="6" t="n">
+      <c r="P11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="P11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="Q11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
@@ -1228,10 +1230,10 @@
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>6</v>
@@ -1267,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
@@ -1282,32 +1284,32 @@
         <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P12" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="W12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1340,45 +1342,45 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="N13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="6" t="inlineStr"/>
-      <c r="U13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="inlineStr"/>
+      <c r="T13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" s="6" t="inlineStr"/>
+      <c r="V13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1411,10 +1413,10 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
@@ -1423,7 +1425,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>2</v>
@@ -1435,22 +1437,22 @@
         <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>9</v>
@@ -1484,46 +1486,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="L15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="M15" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="P15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q15" s="6" t="n">
+      <c r="S15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="R15" s="6" t="n">
+      <c r="T15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>17</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>11</v>
@@ -1562,12 +1564,14 @@
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>1</v>
@@ -1581,9 +1585,7 @@
       <c r="U16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="V16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1648,9 +1650,7 @@
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
@@ -1678,16 +1678,16 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -1728,34 +1728,34 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="L19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>2</v>
@@ -1764,11 +1764,9 @@
         <v>2</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1798,31 +1796,31 @@
         <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>1</v>
@@ -1831,7 +1829,7 @@
         <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1870,22 +1868,22 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>18</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>12</v>
@@ -1894,22 +1892,22 @@
         <v>12</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>8</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>6</v>
@@ -1941,46 +1939,46 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>90</v>
@@ -2030,7 +2028,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-26</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-27</t>
         </is>
       </c>
     </row>
@@ -2072,77 +2070,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -2171,46 +2169,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>23</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>16</v>
@@ -2244,43 +2242,43 @@
         <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>12</v>
@@ -2311,46 +2309,46 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2381,9 +2379,7 @@
       <c r="H7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
@@ -2394,7 +2390,9 @@
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
       <c r="S7" s="6" t="inlineStr"/>
-      <c r="T7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2427,46 +2425,46 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>1</v>
@@ -2495,7 +2493,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>4</v>
@@ -2507,7 +2505,7 @@
         <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
@@ -2568,7 +2566,7 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>4</v>
@@ -2577,22 +2575,22 @@
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
@@ -2604,7 +2602,7 @@
         <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>4</v>
@@ -2644,37 +2642,37 @@
         <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="M11" s="10" t="n">
+      <c r="R11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>47</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>50</v>
@@ -2705,46 +2703,46 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-28)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-27</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-28</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -754,46 +754,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>8</v>
@@ -827,43 +827,43 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>23</v>
@@ -902,46 +902,46 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>6</v>
@@ -973,49 +973,49 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="S8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="V8" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1046,48 +1046,48 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="W9" s="6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="V9" s="6" t="inlineStr"/>
+      <c r="W9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1118,45 +1118,47 @@
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>5</v>
@@ -1192,28 +1194,28 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="K11" s="6" t="n">
+      <c r="L11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N11" s="6" t="n">
+      <c r="O11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
@@ -1225,10 +1227,10 @@
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>6</v>
@@ -1267,10 +1269,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
@@ -1279,33 +1281,31 @@
         <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V12" s="4" t="inlineStr"/>
       <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1341,37 +1341,37 @@
         <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="inlineStr"/>
-      <c r="T13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="6" t="inlineStr"/>
+      <c r="U13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V13" s="6" t="n">
         <v>1</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>5</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
@@ -1418,7 +1418,7 @@
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>2</v>
@@ -1430,25 +1430,25 @@
         <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>5</v>
@@ -1482,46 +1482,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="L15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>11</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>8</v>
@@ -1559,12 +1559,14 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>1</v>
@@ -1578,9 +1580,7 @@
       <c r="T16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
     </row>
@@ -1643,9 +1643,7 @@
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
@@ -1673,16 +1671,16 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
@@ -1724,31 +1722,31 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J19" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J19" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="K19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>2</v>
@@ -1757,12 +1755,12 @@
         <v>2</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
+      <c r="V19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1791,31 +1789,31 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>1</v>
@@ -1824,13 +1822,13 @@
         <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
@@ -1869,16 +1867,16 @@
         <v>18</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>12</v>
@@ -1887,25 +1885,25 @@
         <v>12</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>8</v>
       </c>
       <c r="U21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V21" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="V21" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>8</v>
@@ -1937,46 +1935,46 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>109</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>82</v>
@@ -2026,7 +2024,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-27</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2068,77 +2066,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2170,43 +2168,43 @@
         <v>23</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>15</v>
@@ -2237,43 +2235,43 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>12</v>
@@ -2322,31 +2320,31 @@
         <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2374,9 +2372,7 @@
       <c r="G7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
@@ -2387,7 +2383,9 @@
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2423,46 +2421,46 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="L8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
@@ -2500,7 +2498,7 @@
         <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
@@ -2561,7 +2559,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>4</v>
@@ -2570,22 +2568,22 @@
         <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
@@ -2597,7 +2595,7 @@
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2637,40 +2635,40 @@
         <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="L11" s="10" t="n">
+      <c r="Q11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>47</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>44</v>
@@ -2701,46 +2699,46 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>109</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>82</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-29)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-28</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-29</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>3</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,46 +754,46 @@
         <v>7</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>4</v>
@@ -827,46 +827,46 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>23</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>19</v>
@@ -902,47 +902,45 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>6</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
@@ -971,49 +969,49 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="R8" s="4" t="n">
+      <c r="U8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1047,41 +1045,39 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U9" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="6" t="inlineStr"/>
     </row>
@@ -1115,49 +1111,49 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1190,25 +1186,25 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M11" s="6" t="n">
+      <c r="N11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>7</v>
@@ -1220,16 +1216,16 @@
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>8</v>
@@ -1265,7 +1261,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
@@ -1274,37 +1270,35 @@
         <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V12" s="4" t="inlineStr"/>
-      <c r="W12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1336,42 +1330,42 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6" t="inlineStr"/>
-      <c r="S13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="6" t="inlineStr"/>
+      <c r="T13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>2</v>
@@ -1413,7 +1407,7 @@
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
@@ -1425,31 +1419,31 @@
         <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1480,46 +1474,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="K15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>6</v>
@@ -1556,12 +1550,14 @@
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>1</v>
@@ -1575,9 +1571,7 @@
       <c r="S16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
@@ -1638,9 +1632,7 @@
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
@@ -1668,16 +1660,16 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -1720,28 +1712,28 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>2</v>
@@ -1750,12 +1742,12 @@
         <v>2</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr"/>
+      <c r="U19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1790,25 +1782,25 @@
         <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>1</v>
@@ -1817,13 +1809,13 @@
         <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
@@ -1862,16 +1854,16 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>12</v>
@@ -1880,28 +1872,28 @@
         <v>12</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>8</v>
       </c>
       <c r="T21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U21" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="U21" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="V21" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>6</v>
@@ -1936,43 +1928,43 @@
         <v>109</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>72</v>
@@ -2022,7 +2014,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-28</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-29</t>
         </is>
       </c>
     </row>
@@ -2064,77 +2056,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
@@ -2163,46 +2155,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="R4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>12</v>
@@ -2233,46 +2225,46 @@
         <v>10</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
@@ -2315,34 +2307,34 @@
         <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>1</v>
@@ -2380,7 +2372,9 @@
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2419,43 +2413,43 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>2</v>
@@ -2493,7 +2487,7 @@
         <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
@@ -2526,7 +2520,7 @@
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2563,22 +2557,22 @@
         <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
@@ -2590,13 +2584,13 @@
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>3</v>
@@ -2630,43 +2624,43 @@
         <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="K11" s="10" t="n">
+      <c r="P11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>47</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>39</v>
@@ -2700,43 +2694,43 @@
         <v>109</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>72</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-07-30)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-07-29</t>
+          <t>Evolución abiertas SAT por estado — 2026-07-30</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
@@ -682,46 +682,46 @@
         <v>3</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
+      <c r="T4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -757,40 +757,40 @@
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>10</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>4</v>
@@ -827,46 +827,46 @@
         <v>28</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>18</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>14</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>23</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>16</v>
@@ -902,45 +902,45 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="V7" s="6" t="inlineStr"/>
+      <c r="U7" s="6" t="inlineStr"/>
+      <c r="V7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="W7" s="6" t="n">
         <v>3</v>
       </c>
@@ -971,46 +971,46 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="T8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>10</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>8</v>
@@ -1044,41 +1044,39 @@
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" s="6" t="inlineStr"/>
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="6" t="inlineStr"/>
@@ -1113,43 +1111,43 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1188,22 +1186,22 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="L11" s="6" t="n">
+      <c r="M11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>12</v>
-      </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
@@ -1215,19 +1213,19 @@
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1269,39 +1267,39 @@
         <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U12" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1334,45 +1332,45 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6" t="inlineStr"/>
-      <c r="R13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr"/>
+      <c r="S13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1408,7 +1406,7 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
@@ -1420,31 +1418,31 @@
         <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>4</v>
@@ -1478,46 +1476,46 @@
         <v>1</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N15" s="6" t="n">
+      <c r="U15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>12</v>
@@ -1553,12 +1551,14 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>1</v>
@@ -1572,9 +1572,7 @@
       <c r="R16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
@@ -1633,9 +1631,7 @@
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
@@ -1670,9 +1666,7 @@
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1716,25 +1710,25 @@
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>2</v>
@@ -1743,17 +1737,17 @@
         <v>2</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W19" s="6" t="n">
         <v>3</v>
@@ -1783,25 +1777,25 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1</v>
@@ -1810,13 +1804,13 @@
         <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
@@ -1858,13 +1852,13 @@
         <v>18</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>12</v>
@@ -1873,31 +1867,31 @@
         <v>12</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>8</v>
       </c>
       <c r="S21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T21" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="T21" s="6" t="n">
+      <c r="U21" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="U21" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="V21" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>9</v>
@@ -1929,49 +1923,49 @@
         <v>85</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="U22" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="V22" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="W22" s="8" t="n">
         <v>82</v>
-      </c>
-      <c r="V22" s="8" t="n">
-        <v>72</v>
-      </c>
-      <c r="W22" s="8" t="n">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2018,7 +2012,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-07-29</t>
+          <t>Evolución abiertas SAT por cadena — 2026-07-30</t>
         </is>
       </c>
     </row>
@@ -2060,77 +2054,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
@@ -2159,46 +2153,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>22</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>13</v>
@@ -2232,46 +2226,46 @@
         <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="U5" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="V5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2308,37 +2302,37 @@
         <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2375,7 +2369,9 @@
       <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R7" s="6" t="n">
         <v>1</v>
       </c>
@@ -2417,46 +2413,46 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -2488,7 +2484,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
@@ -2521,7 +2517,7 @@
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2558,22 +2554,22 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
@@ -2585,16 +2581,16 @@
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>4</v>
@@ -2625,46 +2621,46 @@
         <v>35</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="J11" s="10" t="n">
+      <c r="O11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>47</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>41</v>
@@ -2695,49 +2691,49 @@
         <v>85</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <